<commit_message>
Qwen no RAG changes
</commit_message>
<xml_diff>
--- a/artifacts/response_outputs/qwen14b_no_rag.xlsx
+++ b/artifacts/response_outputs/qwen14b_no_rag.xlsx
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,117 +420,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>q_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>question</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>expected_answer</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>resolved_model_name</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>mode</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>prompt_used</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>model_response</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>knowledge_source_data</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>pretrained_data</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>local_context_used</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>web_context_used</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>combined_context_used</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>local_chunk_ids</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>local_chunk_sources</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>local_chunk_texts</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>tavily_chunk_ids</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>tavily_chunk_sources</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>tavily_chunk_texts</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>doc_citations</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>web_citations</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
@@ -551,7 +539,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -587,19 +575,23 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>I don't know the specific Tier 1 and Tier 2 suppliers for EV battery packs operating exclusively in Georgia and Alabama based on my current knowledge. However, I can provide a general approach to identifying such companies:
-- Research major automotive manufacturers with plants in Georgia and Alabama.
-- Identify their primary battery pack suppliers (Tier 1).
-- Look into the supply chains of these Tier 1 suppliers for Tier 2 components and materials.</t>
+          <t>- Panasonic operates as a Tier 1 supplier for Tesla's EV battery packs, though its primary U.S. facility is in Nevada rather than Georgia or Alabama.
+- SK Innovation (now known as SK On) has significant operations in Georgia with a large battery plant near Atlanta, making it a key Tier 1 supplier for several automakers including Ford and Volkswagen.
+- Samsung SDI operates a Tier 1 EV battery manufacturing facility in Birmingham, Alabama, supplying batteries to various automotive companies.
+- LG Energy Solution is another major player as a Tier 1 supplier but its U.S. operations are primarily located in Michigan rather than Georgia or Alabama.
+- POSCO Chemical, a subsidiary of POSCO Group, acts as a Tier 2 supplier providing battery materials for SK On and other manufacturers with facilities potentially supporting their parent company’s activities in the Southeastern U.S.
+- CATL (Contemporary Amperex Technology Ltd.), while expanding globally, currently does not have direct operations in Georgia or Alabama but supplies through partnerships that may include local suppliers.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>I don't know the specific Tier 1 and Tier 2 suppliers for EV battery packs operating exclusively in Georgia and Alabama based on my current knowledge. However, I can provide a general approach to identifying such companies:
-- Research major automotive manufacturers with plants in Georgia and Alabama.
-- Identify their primary battery pack suppliers (Tier 1).
-- Look into the supply chains of these Tier 1 suppliers for Tier 2 components and materials.</t>
+          <t>- Panasonic operates as a Tier 1 supplier for Tesla's EV battery packs, though its primary U.S. facility is in Nevada rather than Georgia or Alabama.
+- SK Innovation (now known as SK On) has significant operations in Georgia with a large battery plant near Atlanta, making it a key Tier 1 supplier for several automakers including Ford and Volkswagen.
+- Samsung SDI operates a Tier 1 EV battery manufacturing facility in Birmingham, Alabama, supplying batteries to various automotive companies.
+- LG Energy Solution is another major player as a Tier 1 supplier but its U.S. operations are primarily located in Michigan rather than Georgia or Alabama.
+- POSCO Chemical, a subsidiary of POSCO Group, acts as a Tier 2 supplier providing battery materials for SK On and other manufacturers with facilities potentially supporting their parent company’s activities in the Southeastern U.S.
+- CATL (Contemporary Amperex Technology Ltd.), while expanding globally, currently does not have direct operations in Georgia or Alabama but supplies through partnerships that may include local suppliers.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -615,14 +607,14 @@
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:10.013180Z</t>
+          <t>2026-03-23T18:20:42.453143Z</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,13 +650,21 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>I don't know. The specific map of suppliers producing power electronics for Battery Electric Vehicles (BEVs) in the Southeast region is not within my current knowledge base. To provide accurate information, I would need to research and verify details about companies operating in that sector and location.</t>
+          <t>- Cree Wolfspeed (North Carolina) - Known for silicon carbide semiconductors used in electric vehicle inverters.
+- Infineon Technologies (Georgia Operations) - Produces a range of power electronics components suitable for BEV applications.
+- ON Semiconductor (Tennessee Operations) - Engages in manufacturing power management ICs and discrete devices relevant to BEVs.
+- Texas Instruments (Texas, near Southeast) - Offers motor driver ICs and other power electronics used in electric vehicles.
+- STMicroelectronics (Georgia Operations) - Provides a variety of power modules and IGBTs for automotive applications.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>I don't know. The specific map of suppliers producing power electronics for Battery Electric Vehicles (BEVs) in the Southeast region is not within my current knowledge base. To provide accurate information, I would need to research and verify details about companies operating in that sector and location.</t>
+          <t>- Cree Wolfspeed (North Carolina) - Known for silicon carbide semiconductors used in electric vehicle inverters.
+- Infineon Technologies (Georgia Operations) - Produces a range of power electronics components suitable for BEV applications.
+- ON Semiconductor (Tennessee Operations) - Engages in manufacturing power management ICs and discrete devices relevant to BEVs.
+- Texas Instruments (Texas, near Southeast) - Offers motor driver ICs and other power electronics used in electric vehicles.
+- STMicroelectronics (Georgia Operations) - Provides a variety of power modules and IGBTs for automotive applications.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -680,14 +680,14 @@
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:11.158956Z</t>
+          <t>2026-03-23T18:20:44.690618Z</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -723,13 +723,19 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>I don't know. The question requires specific regional information about battery manufacturing companies which I do not have without accessing external data sources.</t>
+          <t>- Panasonic manufactures battery modules for Tesla at its Nevada Gigafactory.
+- LG Energy Solution produces both battery modules and complete packs for various automakers, including General Motors and Hyundai-Kia.
+- CATL (Contemporary Amperex Technology Ltd) specializes in manufacturing complete battery packs but also supplies modules to companies like Volkswagen.
+- Samsung SDI is known for producing battery modules that are assembled into packs by automotive manufacturers such as BMW and Renault-Nissan-Mitsubishi alliance.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>I don't know. The question requires specific regional information about battery manufacturing companies which I do not have without accessing external data sources.</t>
+          <t>- Panasonic manufactures battery modules for Tesla at its Nevada Gigafactory.
+- LG Energy Solution produces both battery modules and complete packs for various automakers, including General Motors and Hyundai-Kia.
+- CATL (Contemporary Amperex Technology Ltd) specializes in manufacturing complete battery packs but also supplies modules to companies like Volkswagen.
+- Samsung SDI is known for producing battery modules that are assembled into packs by automotive manufacturers such as BMW and Renault-Nissan-Mitsubishi alliance.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -745,14 +751,14 @@
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:11.770946Z</t>
+          <t>2026-03-23T18:20:46.463003Z</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -788,23 +794,23 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>I don't know specific Southeast-based suppliers capable of producing high-voltage connectors at automotive scale from my current knowledge base. However, here are some general steps one might take to find such suppliers:
-- Research industry directories and databases focusing on Southeast Asian countries.
-- Attend trade shows and conferences related to the automotive industry in Southeast Asia.
-- Contact local business associations or chambers of commerce in relevant Southeast Asian cities.
-- Use online platforms like LinkedIn or specialized B2B networks to connect with manufacturers.
-- Look into government-sponsored export-import websites for Southeast Asian nations.</t>
+          <t>- TE Connectivity in Harrisburg, Texas
+- Molex (a Littelfuse company) with facilities in Irving, Texas
+- Sumitomo Electric Industries with a U.S. base in Plymouth Township, Michigan (near Southeast region)
+- Amphenol Corporation with operations in Atlanta, Georgia
+- Delphi Technologies (now part of Aptiv) has a presence in Troy, Michigan (Southeast proximity)
+- Fujikura Ltd., which operates in Novi, Michigan (close to the Southeast automotive industry hub)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>I don't know specific Southeast-based suppliers capable of producing high-voltage connectors at automotive scale from my current knowledge base. However, here are some general steps one might take to find such suppliers:
-- Research industry directories and databases focusing on Southeast Asian countries.
-- Attend trade shows and conferences related to the automotive industry in Southeast Asia.
-- Contact local business associations or chambers of commerce in relevant Southeast Asian cities.
-- Use online platforms like LinkedIn or specialized B2B networks to connect with manufacturers.
-- Look into government-sponsored export-import websites for Southeast Asian nations.</t>
+          <t>- TE Connectivity in Harrisburg, Texas
+- Molex (a Littelfuse company) with facilities in Irving, Texas
+- Sumitomo Electric Industries with a U.S. base in Plymouth Township, Michigan (near Southeast region)
+- Amphenol Corporation with operations in Atlanta, Georgia
+- Delphi Technologies (now part of Aptiv) has a presence in Troy, Michigan (Southeast proximity)
+- Fujikura Ltd., which operates in Novi, Michigan (close to the Southeast automotive industry hub)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -820,14 +826,14 @@
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:13.815650Z</t>
+          <t>2026-03-23T18:20:48.444272Z</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -863,25 +869,21 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>I don't know the specific current supplier list for DC fast charging hardware with existing OEM (Original Equipment Manufacturer) contracts. However, some well-known companies in this field include:
-- ABB
-- ChargePoint
-- EVBox
-- Triton (formerly SemaConnect)
-- Wallbox
-These companies are known to be involved in manufacturing and supplying DC fast charging solutions for electric vehicles. For the most accurate and up-to-date information regarding OEM contracts, it would be best to consult their official websites or contact them directly.</t>
+          <t>- ABB Ltd manufactures DC fast charging stations and has contracts with various automakers like BMW, Volkswagen, and Daimler.
+- ChargePoint is a major supplier of EV charging solutions including DC fast chargers and works closely with Ford and other car manufacturers.
+- Eaton Corporation supplies high-power DC charging systems and collaborates with OEMs such as General Motors for fleet vehicles.
+- Schneider Electric produces robust DC fast charging hardware and has partnerships with Renault-Nissan-Mitsubishi Alliance.
+- Siemens Energy offers scalable EV charging solutions, including DC fast chargers, and partners with multiple automakers globally.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>I don't know the specific current supplier list for DC fast charging hardware with existing OEM (Original Equipment Manufacturer) contracts. However, some well-known companies in this field include:
-- ABB
-- ChargePoint
-- EVBox
-- Triton (formerly SemaConnect)
-- Wallbox
-These companies are known to be involved in manufacturing and supplying DC fast charging solutions for electric vehicles. For the most accurate and up-to-date information regarding OEM contracts, it would be best to consult their official websites or contact them directly.</t>
+          <t>- ABB Ltd manufactures DC fast charging stations and has contracts with various automakers like BMW, Volkswagen, and Daimler.
+- ChargePoint is a major supplier of EV charging solutions including DC fast chargers and works closely with Ford and other car manufacturers.
+- Eaton Corporation supplies high-power DC charging systems and collaborates with OEMs such as General Motors for fleet vehicles.
+- Schneider Electric produces robust DC fast charging hardware and has partnerships with Renault-Nissan-Mitsubishi Alliance.
+- Siemens Energy offers scalable EV charging solutions, including DC fast chargers, and partners with multiple automakers globally.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -897,14 +899,14 @@
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:15.792900Z</t>
+          <t>2026-03-23T18:20:50.625934Z</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -940,19 +942,21 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>I don't know. The specific list of Tier 2 suppliers for autonomous vehicle sensor systems can change frequently and requires up-to-date industry information to provide accurately. However, generally speaking, some companies that might fit this category include:
-- I don't have precise current data but historically companies like Aptiv (formerly Delphi) could be considered.
-- Other potential players might include companies specializing in electronics manufacturing services (EMS).
-- Tier 2 suppliers often deal with components rather than complete systems, so they would supply parts to the main sensor manufacturers.</t>
+          <t>- BOSCH: Supplies radar and lidar sensors for autonomous driving.
+- Aptiv (formerly Delphi): Provides advanced driver assistance system components including radar and camera-based solutions.
+- Continental AG: Develops a range of ADAS and autonomous driving sensors, including radar and cameras.
+- Veoneer: Offers sensor fusion systems combining data from multiple types of sensors like radars and cameras.
+- Denso Corporation: Engages in the development of various automotive electronics, including advanced sensing technologies.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>I don't know. The specific list of Tier 2 suppliers for autonomous vehicle sensor systems can change frequently and requires up-to-date industry information to provide accurately. However, generally speaking, some companies that might fit this category include:
-- I don't have precise current data but historically companies like Aptiv (formerly Delphi) could be considered.
-- Other potential players might include companies specializing in electronics manufacturing services (EMS).
-- Tier 2 suppliers often deal with components rather than complete systems, so they would supply parts to the main sensor manufacturers.</t>
+          <t>- BOSCH: Supplies radar and lidar sensors for autonomous driving.
+- Aptiv (formerly Delphi): Provides advanced driver assistance system components including radar and camera-based solutions.
+- Continental AG: Develops a range of ADAS and autonomous driving sensors, including radar and cameras.
+- Veoneer: Offers sensor fusion systems combining data from multiple types of sensors like radars and cameras.
+- Denso Corporation: Engages in the development of various automotive electronics, including advanced sensing technologies.</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
@@ -968,14 +972,14 @@
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:17.817605Z</t>
+          <t>2026-03-23T18:20:52.484120Z</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1011,21 +1015,21 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>I don't know. The question requires specific data on electric vehicle (EV) supply chains and supplier concentrations in the Southeast region, which isn't available from my general knowledge alone. However, typically high-risk components might include:
-- Batteries/cells: Due to limited production facilities.
-- Rare earth metals: Essential for magnets and other EV parts with few suppliers globally.
-- Semiconductors: Critical for vehicle electronics but often subject to global shortages.
-- Lithium-ion materials: Key ingredients in batteries that are sourced from a small number of countries.</t>
+          <t>- Battery cells and modules have high supplier concentration risks due to limited production facilities in the region.
+- Electric motors face similar challenges, with few manufacturers specializing in their production.
+- Power electronics and management systems also exhibit significant supply chain risks because of a lack of local suppliers.
+- Rare earth materials used in EV components are at risk due to reliance on imports from China.
+- Lithium-ion battery raw materials present high concentration risks owing to limited regional sourcing options.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>I don't know. The question requires specific data on electric vehicle (EV) supply chains and supplier concentrations in the Southeast region, which isn't available from my general knowledge alone. However, typically high-risk components might include:
-- Batteries/cells: Due to limited production facilities.
-- Rare earth metals: Essential for magnets and other EV parts with few suppliers globally.
-- Semiconductors: Critical for vehicle electronics but often subject to global shortages.
-- Lithium-ion materials: Key ingredients in batteries that are sourced from a small number of countries.</t>
+          <t>- Battery cells and modules have high supplier concentration risks due to limited production facilities in the region.
+- Electric motors face similar challenges, with few manufacturers specializing in their production.
+- Power electronics and management systems also exhibit significant supply chain risks because of a lack of local suppliers.
+- Rare earth materials used in EV components are at risk due to reliance on imports from China.
+- Lithium-ion battery raw materials present high concentration risks owing to limited regional sourcing options.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -1041,14 +1045,14 @@
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:19.866867Z</t>
+          <t>2026-03-23T18:20:54.202886Z</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1084,25 +1088,23 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>- Dependency on cobalt from Congo for lithium-ion batteries
-- Reliance on lithium from Australia and Chile for battery production
-- Nickel sourcing from Indonesia and Philippines crucial for battery efficiency
-- Manganese imports from South Africa and China impact battery cost and performance
-- Graphite supply from China dominates the market, affecting availability and pricing
-- Rare earth elements from China are vital for magnet production in electric vehicles
-- Trade policies and geopolitical tensions can disrupt material flows globally</t>
+          <t>- Many electric vehicle (EV) manufacturers rely heavily on imported lithium from countries like Chile, Australia, and China for battery production.
+- Cobalt, another critical component in batteries, is predominantly sourced from the Democratic Republic of Congo due to its rich deposits.
+- Supply chain disruptions in these regions can significantly impact battery manufacturing capacity globally.
+- The geopolitical tensions between major importing nations and exporting countries affect supply stability and pricing.
+- Diversification efforts are underway by companies to secure alternative sources and reduce dependency on single-country imports.
+- Recycling initiatives for spent batteries aim to create a more sustainable and less dependent supply chain in the long term.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>- Dependency on cobalt from Congo for lithium-ion batteries
-- Reliance on lithium from Australia and Chile for battery production
-- Nickel sourcing from Indonesia and Philippines crucial for battery efficiency
-- Manganese imports from South Africa and China impact battery cost and performance
-- Graphite supply from China dominates the market, affecting availability and pricing
-- Rare earth elements from China are vital for magnet production in electric vehicles
-- Trade policies and geopolitical tensions can disrupt material flows globally</t>
+          <t>- Many electric vehicle (EV) manufacturers rely heavily on imported lithium from countries like Chile, Australia, and China for battery production.
+- Cobalt, another critical component in batteries, is predominantly sourced from the Democratic Republic of Congo due to its rich deposits.
+- Supply chain disruptions in these regions can significantly impact battery manufacturing capacity globally.
+- The geopolitical tensions between major importing nations and exporting countries affect supply stability and pricing.
+- Diversification efforts are underway by companies to secure alternative sources and reduce dependency on single-country imports.
+- Recycling initiatives for spent batteries aim to create a more sustainable and less dependent supply chain in the long term.</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -1118,14 +1120,14 @@
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:21.614629Z</t>
+          <t>2026-03-23T18:20:56.503286Z</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1161,21 +1163,23 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>I don't know. However, based on general manufacturing and supply chain knowledge:
-- **Supply Chain Disruptions:** Issues in the procurement of components from secondary suppliers can lead to delays in OEM (Original Equipment Manufacturer) production lines.
-- **Component Shortages:** If a Tier 2 or Tier 3 supplier faces difficulties producing critical parts, it could cause shortages that ripple up to the OEMs.
-- **Quality Control Problems:** Lower-tier suppliers might experience quality control issues affecting the reliability of components supplied to OEMs.
-- **Logistical Challenges:** Transportation and warehousing problems at lower tiers can disrupt the timely delivery of materials needed by OEMs.</t>
+          <t>- Tier 2 and Tier 3 bottlenecks can significantly affect the supply chain efficiency of Original Equipment Manufacturers (OEMs).
+- Delays in obtaining components from Tier 2 suppliers can lead to reduced output at assembly lines, impacting overall production schedules.
+- Quality issues with Tier 3 parts can cascade up through the supply chain, causing rework and delays for OEMs.
+- Shortages or disruptions in raw materials supplied by Tier 3 vendors can limit the availability of critical components needed by Tier 2 suppliers.
+- Inflexible logistics from Tier 2 and Tier 3 suppliers can cause bottlenecks in inventory management at OEM facilities.
+- Communication breakdowns between lower-tier suppliers and OEMs can result in mismatches in production forecasts, leading to excess or shortage issues.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>I don't know. However, based on general manufacturing and supply chain knowledge:
-- **Supply Chain Disruptions:** Issues in the procurement of components from secondary suppliers can lead to delays in OEM (Original Equipment Manufacturer) production lines.
-- **Component Shortages:** If a Tier 2 or Tier 3 supplier faces difficulties producing critical parts, it could cause shortages that ripple up to the OEMs.
-- **Quality Control Problems:** Lower-tier suppliers might experience quality control issues affecting the reliability of components supplied to OEMs.
-- **Logistical Challenges:** Transportation and warehousing problems at lower tiers can disrupt the timely delivery of materials needed by OEMs.</t>
+          <t>- Tier 2 and Tier 3 bottlenecks can significantly affect the supply chain efficiency of Original Equipment Manufacturers (OEMs).
+- Delays in obtaining components from Tier 2 suppliers can lead to reduced output at assembly lines, impacting overall production schedules.
+- Quality issues with Tier 3 parts can cascade up through the supply chain, causing rework and delays for OEMs.
+- Shortages or disruptions in raw materials supplied by Tier 3 vendors can limit the availability of critical components needed by Tier 2 suppliers.
+- Inflexible logistics from Tier 2 and Tier 3 suppliers can cause bottlenecks in inventory management at OEM facilities.
+- Communication breakdowns between lower-tier suppliers and OEMs can result in mismatches in production forecasts, leading to excess or shortage issues.</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -1191,14 +1195,14 @@
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:23.981284Z</t>
+          <t>2026-03-23T18:20:59.393016Z</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1234,13 +1238,21 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>I don't know. The specific growth rates of electric vehicle (EV) supply chain segments in the Southeast can vary based on recent investments, government policies, and market demands which I do not have current data for. To provide accurate information would require up-to-date industry reports or analysis focusing specifically on that region.</t>
+          <t>- Battery manufacturing and recycling facilities are expanding rapidly due to proximity to automotive assembly plants.
+- Charging infrastructure installation companies are seeing significant growth as electric vehicle adoption increases.
+- Lithium-ion battery component suppliers are establishing regional hubs for quicker delivery times.
+- Electric vehicle (EV) service centers specializing in EV maintenance and repair are proliferating.
+- Regional distribution networks for EV parts and components are becoming more efficient and extensive.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>I don't know. The specific growth rates of electric vehicle (EV) supply chain segments in the Southeast can vary based on recent investments, government policies, and market demands which I do not have current data for. To provide accurate information would require up-to-date industry reports or analysis focusing specifically on that region.</t>
+          <t>- Battery manufacturing and recycling facilities are expanding rapidly due to proximity to automotive assembly plants.
+- Charging infrastructure installation companies are seeing significant growth as electric vehicle adoption increases.
+- Lithium-ion battery component suppliers are establishing regional hubs for quicker delivery times.
+- Electric vehicle (EV) service centers specializing in EV maintenance and repair are proliferating.
+- Regional distribution networks for EV parts and components are becoming more efficient and extensive.</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -1256,14 +1268,14 @@
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:25.204609Z</t>
+          <t>2026-03-23T18:21:00.957549Z</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1299,21 +1311,21 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>I don't know which specific companies are currently making a definitive shift from internal combustion engine (ICE) components to electric vehicle (EV)-focused products. However, here are some general trends and examples:
-- Many automotive suppliers are diversifying their product lines to include more EV-related parts.
-- Companies like Bosch and Continental have been investing in electrification technologies.
-- Some companies might be reducing ICE component production while increasing EV part manufacturing.
-- There could be a trend among smaller specialized firms focusing solely on EV components.</t>
+          <t>- Volkswagen has committed significant resources to electric vehicle production and is phasing out traditional internal combustion engine (ICE) vehicles in many markets.
+- General Motors is investing heavily in battery technology and plans to launch multiple new electric models, reducing focus on conventional engines.
+- Ford Motor Company is expanding its EV lineup with the Mustang Mach-E and F-150 Lightning while scaling back some ICE vehicle production lines.
+- Toyota has announced a shift towards hybrid and fully electric vehicles as part of its long-term strategy, though it continues to support traditional ICE technology in certain markets.
+- Hyundai-Kia is rapidly growing its portfolio of electric cars and plans substantial investments in battery manufacturing facilities.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>I don't know which specific companies are currently making a definitive shift from internal combustion engine (ICE) components to electric vehicle (EV)-focused products. However, here are some general trends and examples:
-- Many automotive suppliers are diversifying their product lines to include more EV-related parts.
-- Companies like Bosch and Continental have been investing in electrification technologies.
-- Some companies might be reducing ICE component production while increasing EV part manufacturing.
-- There could be a trend among smaller specialized firms focusing solely on EV components.</t>
+          <t>- Volkswagen has committed significant resources to electric vehicle production and is phasing out traditional internal combustion engine (ICE) vehicles in many markets.
+- General Motors is investing heavily in battery technology and plans to launch multiple new electric models, reducing focus on conventional engines.
+- Ford Motor Company is expanding its EV lineup with the Mustang Mach-E and F-150 Lightning while scaling back some ICE vehicle production lines.
+- Toyota has announced a shift towards hybrid and fully electric vehicles as part of its long-term strategy, though it continues to support traditional ICE technology in certain markets.
+- Hyundai-Kia is rapidly growing its portfolio of electric cars and plans substantial investments in battery manufacturing facilities.</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
@@ -1329,14 +1341,14 @@
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:27.104582Z</t>
+          <t>2026-03-23T18:21:03.409028Z</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1372,19 +1384,23 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>I don't know. The regional changes in demand for battery manufacturing equipment are influenced by various factors such as government policies, technological advancements, and market trends which I do not have current data on to provide specific insights. However, generally speaking:
-- Asia-Pacific regions like China and South Korea are seeing high growth due to strong government support and large-scale investments.
-- Europe is also experiencing increased demand driven by ambitious green energy targets and automotive electrification initiatives.
-- North America is witnessing steady growth but may lag behind Asia-Pacific in terms of scale and speed.</t>
+          <t>- Demand for battery manufacturing equipment is increasing in Asia due to the rapid growth of electric vehicle (EV) markets and government incentives in countries like China and South Korea.
+- Europe is also seeing significant growth, driven by ambitious climate goals and investments from major automakers such as Volkswagen and BMW.
+- North America is experiencing strong demand, particularly in the United States, where there are substantial federal and state-level initiatives to support EV infrastructure and battery production.
+- Latin American countries like Brazil and Chile are showing interest due to their rich lithium reserves and growing automotive industries.
+- In Africa, regions with significant mineral resources are attracting investments for battery manufacturing as global supply chains diversify.
+- Middle Eastern nations are exploring opportunities in battery manufacturing to reduce reliance on oil exports and capitalize on renewable energy initiatives.</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>I don't know. The regional changes in demand for battery manufacturing equipment are influenced by various factors such as government policies, technological advancements, and market trends which I do not have current data on to provide specific insights. However, generally speaking:
-- Asia-Pacific regions like China and South Korea are seeing high growth due to strong government support and large-scale investments.
-- Europe is also experiencing increased demand driven by ambitious green energy targets and automotive electrification initiatives.
-- North America is witnessing steady growth but may lag behind Asia-Pacific in terms of scale and speed.</t>
+          <t>- Demand for battery manufacturing equipment is increasing in Asia due to the rapid growth of electric vehicle (EV) markets and government incentives in countries like China and South Korea.
+- Europe is also seeing significant growth, driven by ambitious climate goals and investments from major automakers such as Volkswagen and BMW.
+- North America is experiencing strong demand, particularly in the United States, where there are substantial federal and state-level initiatives to support EV infrastructure and battery production.
+- Latin American countries like Brazil and Chile are showing interest due to their rich lithium reserves and growing automotive industries.
+- In Africa, regions with significant mineral resources are attracting investments for battery manufacturing as global supply chains diversify.
+- Middle Eastern nations are exploring opportunities in battery manufacturing to reduce reliance on oil exports and capitalize on renewable energy initiatives.</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -1400,14 +1416,14 @@
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:29.138734Z</t>
+          <t>2026-03-23T18:21:06.279677Z</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1443,13 +1459,21 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>I don't know. The question requires specific data on electric vehicle (EV) supplier density and workforce capacity in Southeast counties, which I do not have access to without external sources or databases.</t>
+          <t>- Miami-Dade County, Florida: High concentration of electric vehicle (EV) suppliers and a large workforce in the automotive industry.
+- Orange County, Florida: Presence of EV charging infrastructure companies and significant employment opportunities in tech and manufacturing sectors.
+- Harris County, Texas: Home to multiple EV component manufacturers and a robust labor market with skilled workers.
+- Maricopa County, Arizona: Growing presence of EV startups and established suppliers, along with a trainable workforce due to local educational institutions.
+- Clark County, Nevada: Increasing number of EV-related businesses and a growing tech-savvy workforce.</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>I don't know. The question requires specific data on electric vehicle (EV) supplier density and workforce capacity in Southeast counties, which I do not have access to without external sources or databases.</t>
+          <t>- Miami-Dade County, Florida: High concentration of electric vehicle (EV) suppliers and a large workforce in the automotive industry.
+- Orange County, Florida: Presence of EV charging infrastructure companies and significant employment opportunities in tech and manufacturing sectors.
+- Harris County, Texas: Home to multiple EV component manufacturers and a robust labor market with skilled workers.
+- Maricopa County, Arizona: Growing presence of EV startups and established suppliers, along with a trainable workforce due to local educational institutions.
+- Clark County, Nevada: Increasing number of EV-related businesses and a growing tech-savvy workforce.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -1465,14 +1489,14 @@
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:29.963294Z</t>
+          <t>2026-03-23T18:21:08.470736Z</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1508,23 +1532,21 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>I don't know. However, I can provide a general approach to identifying such regions:
-- Proximity to major automotive manufacturing hubs
-- Availability of skilled labor force in electronics and manufacturing sectors
-- Presence of established supply chains for raw materials like lithium, cobalt, nickel
-- Government incentives or policies supporting battery production and R&amp;D
-- Access to renewable energy sources for sustainable operations</t>
+          <t>- Southeast Asia: Countries like Thailand, Vietnam, and Indonesia have emerging automotive industries with supportive government policies for electric vehicle (EV) manufacturing.
+- North America: The United States has a robust industrial base and a growing EV market, supported by local supply chains and favorable tax incentives.
+- Europe: Germany and Poland offer established manufacturing ecosystems along with proximity to major car manufacturers and battery suppliers like CATL and LG Energy Solution.
+- China: Despite potential trade barriers, it remains the world's largest EV market with extensive supplier networks and technological advancements in battery technology.
+- South Korea: Home to leading battery companies such as Samsung SDI and LG Chem, providing a strong local supply chain for battery pack assembly.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>I don't know. However, I can provide a general approach to identifying such regions:
-- Proximity to major automotive manufacturing hubs
-- Availability of skilled labor force in electronics and manufacturing sectors
-- Presence of established supply chains for raw materials like lithium, cobalt, nickel
-- Government incentives or policies supporting battery production and R&amp;D
-- Access to renewable energy sources for sustainable operations</t>
+          <t>- Southeast Asia: Countries like Thailand, Vietnam, and Indonesia have emerging automotive industries with supportive government policies for electric vehicle (EV) manufacturing.
+- North America: The United States has a robust industrial base and a growing EV market, supported by local supply chains and favorable tax incentives.
+- Europe: Germany and Poland offer established manufacturing ecosystems along with proximity to major car manufacturers and battery suppliers like CATL and LG Energy Solution.
+- China: Despite potential trade barriers, it remains the world's largest EV market with extensive supplier networks and technological advancements in battery technology.
+- South Korea: Home to leading battery companies such as Samsung SDI and LG Chem, providing a strong local supply chain for battery pack assembly.</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -1540,14 +1562,14 @@
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:31.463702Z</t>
+          <t>2026-03-23T18:21:11.035835Z</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1583,19 +1605,21 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>I don't know the specific locations of all emerging electric vehicle (EV) manufacturing clusters outside of major metropolitan areas with absolute certainty. However, based on general trends and reports, here are a few regions where such activity might be occurring:
-- Southeast Asia: Countries like Thailand and Indonesia have been developing their EV industries.
-- Eastern Europe: Some countries in this region are beginning to establish or expand EV production facilities.
-- Latin America: Certain nations in South America are showing interest in building up their EV manufacturing capabilities.</t>
+          <t>- Rural areas in China are seeing the growth of electric vehicle (EV) manufacturing due to government incentives and infrastructure development.
+- Small cities and towns in India are becoming hubs for EV production as local demand increases and startups enter the market.
+- Eastern European countries like Romania and Bulgaria are attracting EV manufacturers with lower operational costs and supportive policies.
+- In North America, smaller cities such as Windsor, Ontario (near Detroit), are leveraging existing automotive industry infrastructure to develop EV manufacturing capabilities.
+- South Korea is expanding its EV production beyond Seoul and Busan, with new plants being established in secondary cities like Daejeon and Gwangju.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>I don't know the specific locations of all emerging electric vehicle (EV) manufacturing clusters outside of major metropolitan areas with absolute certainty. However, based on general trends and reports, here are a few regions where such activity might be occurring:
-- Southeast Asia: Countries like Thailand and Indonesia have been developing their EV industries.
-- Eastern Europe: Some countries in this region are beginning to establish or expand EV production facilities.
-- Latin America: Certain nations in South America are showing interest in building up their EV manufacturing capabilities.</t>
+          <t>- Rural areas in China are seeing the growth of electric vehicle (EV) manufacturing due to government incentives and infrastructure development.
+- Small cities and towns in India are becoming hubs for EV production as local demand increases and startups enter the market.
+- Eastern European countries like Romania and Bulgaria are attracting EV manufacturers with lower operational costs and supportive policies.
+- In North America, smaller cities such as Windsor, Ontario (near Detroit), are leveraging existing automotive industry infrastructure to develop EV manufacturing capabilities.
+- South Korea is expanding its EV production beyond Seoul and Busan, with new plants being established in secondary cities like Daejeon and Gwangju.</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
@@ -1611,7 +1635,7 @@
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:33.355808Z</t>
+          <t>2026-03-23T18:21:13.371844Z</t>
         </is>
       </c>
     </row>
@@ -1630,82 +1654,82 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>q_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>question</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>resolved_model_name</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>mode</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>prompt_used</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>answer_text</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>error_message</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>timing</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>tokens_in</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>tokens_out</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>tokens_total</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>cost_usd</t>
         </is>
@@ -1714,7 +1738,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1749,10 +1773,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>I don't know the specific Tier 1 and Tier 2 suppliers for EV battery packs operating exclusively in Georgia and Alabama based on my current knowledge. However, I can provide a general approach to identifying such companies:
-- Research major automotive manufacturers with plants in Georgia and Alabama.
-- Identify their primary battery pack suppliers (Tier 1).
-- Look into the supply chains of these Tier 1 suppliers for Tier 2 components and materials.</t>
+          <t>- Panasonic operates as a Tier 1 supplier for Tesla's EV battery packs, though its primary U.S. facility is in Nevada rather than Georgia or Alabama.
+- SK Innovation (now known as SK On) has significant operations in Georgia with a large battery plant near Atlanta, making it a key Tier 1 supplier for several automakers including Ford and Volkswagen.
+- Samsung SDI operates a Tier 1 EV battery manufacturing facility in Birmingham, Alabama, supplying batteries to various automotive companies.
+- LG Energy Solution is another major player as a Tier 1 supplier but its U.S. operations are primarily located in Michigan rather than Georgia or Alabama.
+- POSCO Chemical, a subsidiary of POSCO Group, acts as a Tier 2 supplier providing battery materials for SK On and other manufacturers with facilities potentially supporting their parent company’s activities in the Southeastern U.S.
+- CATL (Contemporary Amperex Technology Ltd.), while expanding globally, currently does not have direct operations in Georgia or Alabama but supplies through partnerships that may include local suppliers.</t>
         </is>
       </c>
       <c r="I2" t="b">
@@ -1761,12 +1787,12 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:10.013180Z</t>
+          <t>2026-03-23T18:20:42.453143Z</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 20640.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 3730.0}</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -1777,7 +1803,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1812,7 +1838,11 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>I don't know. The specific map of suppliers producing power electronics for Battery Electric Vehicles (BEVs) in the Southeast region is not within my current knowledge base. To provide accurate information, I would need to research and verify details about companies operating in that sector and location.</t>
+          <t>- Cree Wolfspeed (North Carolina) - Known for silicon carbide semiconductors used in electric vehicle inverters.
+- Infineon Technologies (Georgia Operations) - Produces a range of power electronics components suitable for BEV applications.
+- ON Semiconductor (Tennessee Operations) - Engages in manufacturing power management ICs and discrete devices relevant to BEVs.
+- Texas Instruments (Texas, near Southeast) - Offers motor driver ICs and other power electronics used in electric vehicles.
+- STMicroelectronics (Georgia Operations) - Provides a variety of power modules and IGBTs for automotive applications.</t>
         </is>
       </c>
       <c r="I3" t="b">
@@ -1821,12 +1851,12 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:11.158956Z</t>
+          <t>2026-03-23T18:20:44.690618Z</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1150.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2240.0}</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -1837,7 +1867,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1872,7 +1902,10 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>I don't know. The question requires specific regional information about battery manufacturing companies which I do not have without accessing external data sources.</t>
+          <t>- Panasonic manufactures battery modules for Tesla at its Nevada Gigafactory.
+- LG Energy Solution produces both battery modules and complete packs for various automakers, including General Motors and Hyundai-Kia.
+- CATL (Contemporary Amperex Technology Ltd) specializes in manufacturing complete battery packs but also supplies modules to companies like Volkswagen.
+- Samsung SDI is known for producing battery modules that are assembled into packs by automotive manufacturers such as BMW and Renault-Nissan-Mitsubishi alliance.</t>
         </is>
       </c>
       <c r="I4" t="b">
@@ -1881,12 +1914,12 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:11.770946Z</t>
+          <t>2026-03-23T18:20:46.463003Z</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 610.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1770.0}</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -1897,7 +1930,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1932,12 +1965,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>I don't know specific Southeast-based suppliers capable of producing high-voltage connectors at automotive scale from my current knowledge base. However, here are some general steps one might take to find such suppliers:
-- Research industry directories and databases focusing on Southeast Asian countries.
-- Attend trade shows and conferences related to the automotive industry in Southeast Asia.
-- Contact local business associations or chambers of commerce in relevant Southeast Asian cities.
-- Use online platforms like LinkedIn or specialized B2B networks to connect with manufacturers.
-- Look into government-sponsored export-import websites for Southeast Asian nations.</t>
+          <t>- TE Connectivity in Harrisburg, Texas
+- Molex (a Littelfuse company) with facilities in Irving, Texas
+- Sumitomo Electric Industries with a U.S. base in Plymouth Township, Michigan (near Southeast region)
+- Amphenol Corporation with operations in Atlanta, Georgia
+- Delphi Technologies (now part of Aptiv) has a presence in Troy, Michigan (Southeast proximity)
+- Fujikura Ltd., which operates in Novi, Michigan (close to the Southeast automotive industry hub)</t>
         </is>
       </c>
       <c r="I5" t="b">
@@ -1946,12 +1979,12 @@
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:13.815650Z</t>
+          <t>2026-03-23T18:20:48.444272Z</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2040.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1980.0}</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1962,7 +1995,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1997,13 +2030,11 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>I don't know the specific current supplier list for DC fast charging hardware with existing OEM (Original Equipment Manufacturer) contracts. However, some well-known companies in this field include:
-- ABB
-- ChargePoint
-- EVBox
-- Triton (formerly SemaConnect)
-- Wallbox
-These companies are known to be involved in manufacturing and supplying DC fast charging solutions for electric vehicles. For the most accurate and up-to-date information regarding OEM contracts, it would be best to consult their official websites or contact them directly.</t>
+          <t>- ABB Ltd manufactures DC fast charging stations and has contracts with various automakers like BMW, Volkswagen, and Daimler.
+- ChargePoint is a major supplier of EV charging solutions including DC fast chargers and works closely with Ford and other car manufacturers.
+- Eaton Corporation supplies high-power DC charging systems and collaborates with OEMs such as General Motors for fleet vehicles.
+- Schneider Electric produces robust DC fast charging hardware and has partnerships with Renault-Nissan-Mitsubishi Alliance.
+- Siemens Energy offers scalable EV charging solutions, including DC fast chargers, and partners with multiple automakers globally.</t>
         </is>
       </c>
       <c r="I6" t="b">
@@ -2012,12 +2043,12 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:15.792900Z</t>
+          <t>2026-03-23T18:20:50.625934Z</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1980.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2180.0}</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -2028,7 +2059,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2063,10 +2094,11 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>I don't know. The specific list of Tier 2 suppliers for autonomous vehicle sensor systems can change frequently and requires up-to-date industry information to provide accurately. However, generally speaking, some companies that might fit this category include:
-- I don't have precise current data but historically companies like Aptiv (formerly Delphi) could be considered.
-- Other potential players might include companies specializing in electronics manufacturing services (EMS).
-- Tier 2 suppliers often deal with components rather than complete systems, so they would supply parts to the main sensor manufacturers.</t>
+          <t>- BOSCH: Supplies radar and lidar sensors for autonomous driving.
+- Aptiv (formerly Delphi): Provides advanced driver assistance system components including radar and camera-based solutions.
+- Continental AG: Develops a range of ADAS and autonomous driving sensors, including radar and cameras.
+- Veoneer: Offers sensor fusion systems combining data from multiple types of sensors like radars and cameras.
+- Denso Corporation: Engages in the development of various automotive electronics, including advanced sensing technologies.</t>
         </is>
       </c>
       <c r="I7" t="b">
@@ -2075,12 +2107,12 @@
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:17.817605Z</t>
+          <t>2026-03-23T18:20:52.484120Z</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2020.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1860.0}</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -2091,7 +2123,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2126,11 +2158,11 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>I don't know. The question requires specific data on electric vehicle (EV) supply chains and supplier concentrations in the Southeast region, which isn't available from my general knowledge alone. However, typically high-risk components might include:
-- Batteries/cells: Due to limited production facilities.
-- Rare earth metals: Essential for magnets and other EV parts with few suppliers globally.
-- Semiconductors: Critical for vehicle electronics but often subject to global shortages.
-- Lithium-ion materials: Key ingredients in batteries that are sourced from a small number of countries.</t>
+          <t>- Battery cells and modules have high supplier concentration risks due to limited production facilities in the region.
+- Electric motors face similar challenges, with few manufacturers specializing in their production.
+- Power electronics and management systems also exhibit significant supply chain risks because of a lack of local suppliers.
+- Rare earth materials used in EV components are at risk due to reliance on imports from China.
+- Lithium-ion battery raw materials present high concentration risks owing to limited regional sourcing options.</t>
         </is>
       </c>
       <c r="I8" t="b">
@@ -2139,12 +2171,12 @@
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:19.866867Z</t>
+          <t>2026-03-23T18:20:54.202886Z</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2050.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1720.0}</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -2155,7 +2187,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2190,13 +2222,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>- Dependency on cobalt from Congo for lithium-ion batteries
-- Reliance on lithium from Australia and Chile for battery production
-- Nickel sourcing from Indonesia and Philippines crucial for battery efficiency
-- Manganese imports from South Africa and China impact battery cost and performance
-- Graphite supply from China dominates the market, affecting availability and pricing
-- Rare earth elements from China are vital for magnet production in electric vehicles
-- Trade policies and geopolitical tensions can disrupt material flows globally</t>
+          <t>- Many electric vehicle (EV) manufacturers rely heavily on imported lithium from countries like Chile, Australia, and China for battery production.
+- Cobalt, another critical component in batteries, is predominantly sourced from the Democratic Republic of Congo due to its rich deposits.
+- Supply chain disruptions in these regions can significantly impact battery manufacturing capacity globally.
+- The geopolitical tensions between major importing nations and exporting countries affect supply stability and pricing.
+- Diversification efforts are underway by companies to secure alternative sources and reduce dependency on single-country imports.
+- Recycling initiatives for spent batteries aim to create a more sustainable and less dependent supply chain in the long term.</t>
         </is>
       </c>
       <c r="I9" t="b">
@@ -2205,12 +2236,12 @@
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:21.614629Z</t>
+          <t>2026-03-23T18:20:56.503286Z</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1750.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2300.0}</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -2221,7 +2252,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2256,11 +2287,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>I don't know. However, based on general manufacturing and supply chain knowledge:
-- **Supply Chain Disruptions:** Issues in the procurement of components from secondary suppliers can lead to delays in OEM (Original Equipment Manufacturer) production lines.
-- **Component Shortages:** If a Tier 2 or Tier 3 supplier faces difficulties producing critical parts, it could cause shortages that ripple up to the OEMs.
-- **Quality Control Problems:** Lower-tier suppliers might experience quality control issues affecting the reliability of components supplied to OEMs.
-- **Logistical Challenges:** Transportation and warehousing problems at lower tiers can disrupt the timely delivery of materials needed by OEMs.</t>
+          <t>- Tier 2 and Tier 3 bottlenecks can significantly affect the supply chain efficiency of Original Equipment Manufacturers (OEMs).
+- Delays in obtaining components from Tier 2 suppliers can lead to reduced output at assembly lines, impacting overall production schedules.
+- Quality issues with Tier 3 parts can cascade up through the supply chain, causing rework and delays for OEMs.
+- Shortages or disruptions in raw materials supplied by Tier 3 vendors can limit the availability of critical components needed by Tier 2 suppliers.
+- Inflexible logistics from Tier 2 and Tier 3 suppliers can cause bottlenecks in inventory management at OEM facilities.
+- Communication breakdowns between lower-tier suppliers and OEMs can result in mismatches in production forecasts, leading to excess or shortage issues.</t>
         </is>
       </c>
       <c r="I10" t="b">
@@ -2269,12 +2301,12 @@
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:23.981284Z</t>
+          <t>2026-03-23T18:20:59.393016Z</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2370.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2890.0}</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -2285,7 +2317,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2320,7 +2352,11 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>I don't know. The specific growth rates of electric vehicle (EV) supply chain segments in the Southeast can vary based on recent investments, government policies, and market demands which I do not have current data for. To provide accurate information would require up-to-date industry reports or analysis focusing specifically on that region.</t>
+          <t>- Battery manufacturing and recycling facilities are expanding rapidly due to proximity to automotive assembly plants.
+- Charging infrastructure installation companies are seeing significant growth as electric vehicle adoption increases.
+- Lithium-ion battery component suppliers are establishing regional hubs for quicker delivery times.
+- Electric vehicle (EV) service centers specializing in EV maintenance and repair are proliferating.
+- Regional distribution networks for EV parts and components are becoming more efficient and extensive.</t>
         </is>
       </c>
       <c r="I11" t="b">
@@ -2329,12 +2365,12 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:25.204609Z</t>
+          <t>2026-03-23T18:21:00.957549Z</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1220.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1560.0}</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -2345,7 +2381,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2380,11 +2416,11 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>I don't know which specific companies are currently making a definitive shift from internal combustion engine (ICE) components to electric vehicle (EV)-focused products. However, here are some general trends and examples:
-- Many automotive suppliers are diversifying their product lines to include more EV-related parts.
-- Companies like Bosch and Continental have been investing in electrification technologies.
-- Some companies might be reducing ICE component production while increasing EV part manufacturing.
-- There could be a trend among smaller specialized firms focusing solely on EV components.</t>
+          <t>- Volkswagen has committed significant resources to electric vehicle production and is phasing out traditional internal combustion engine (ICE) vehicles in many markets.
+- General Motors is investing heavily in battery technology and plans to launch multiple new electric models, reducing focus on conventional engines.
+- Ford Motor Company is expanding its EV lineup with the Mustang Mach-E and F-150 Lightning while scaling back some ICE vehicle production lines.
+- Toyota has announced a shift towards hybrid and fully electric vehicles as part of its long-term strategy, though it continues to support traditional ICE technology in certain markets.
+- Hyundai-Kia is rapidly growing its portfolio of electric cars and plans substantial investments in battery manufacturing facilities.</t>
         </is>
       </c>
       <c r="I12" t="b">
@@ -2393,12 +2429,12 @@
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:27.104582Z</t>
+          <t>2026-03-23T18:21:03.409028Z</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1900.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2450.0}</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -2409,7 +2445,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2444,10 +2480,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>I don't know. The regional changes in demand for battery manufacturing equipment are influenced by various factors such as government policies, technological advancements, and market trends which I do not have current data on to provide specific insights. However, generally speaking:
-- Asia-Pacific regions like China and South Korea are seeing high growth due to strong government support and large-scale investments.
-- Europe is also experiencing increased demand driven by ambitious green energy targets and automotive electrification initiatives.
-- North America is witnessing steady growth but may lag behind Asia-Pacific in terms of scale and speed.</t>
+          <t>- Demand for battery manufacturing equipment is increasing in Asia due to the rapid growth of electric vehicle (EV) markets and government incentives in countries like China and South Korea.
+- Europe is also seeing significant growth, driven by ambitious climate goals and investments from major automakers such as Volkswagen and BMW.
+- North America is experiencing strong demand, particularly in the United States, where there are substantial federal and state-level initiatives to support EV infrastructure and battery production.
+- Latin American countries like Brazil and Chile are showing interest due to their rich lithium reserves and growing automotive industries.
+- In Africa, regions with significant mineral resources are attracting investments for battery manufacturing as global supply chains diversify.
+- Middle Eastern nations are exploring opportunities in battery manufacturing to reduce reliance on oil exports and capitalize on renewable energy initiatives.</t>
         </is>
       </c>
       <c r="I13" t="b">
@@ -2456,12 +2494,12 @@
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:29.138734Z</t>
+          <t>2026-03-23T18:21:06.279677Z</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2030.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2870.0}</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -2472,7 +2510,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2507,7 +2545,11 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>I don't know. The question requires specific data on electric vehicle (EV) supplier density and workforce capacity in Southeast counties, which I do not have access to without external sources or databases.</t>
+          <t>- Miami-Dade County, Florida: High concentration of electric vehicle (EV) suppliers and a large workforce in the automotive industry.
+- Orange County, Florida: Presence of EV charging infrastructure companies and significant employment opportunities in tech and manufacturing sectors.
+- Harris County, Texas: Home to multiple EV component manufacturers and a robust labor market with skilled workers.
+- Maricopa County, Arizona: Growing presence of EV startups and established suppliers, along with a trainable workforce due to local educational institutions.
+- Clark County, Nevada: Increasing number of EV-related businesses and a growing tech-savvy workforce.</t>
         </is>
       </c>
       <c r="I14" t="b">
@@ -2516,12 +2558,12 @@
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:29.963294Z</t>
+          <t>2026-03-23T18:21:08.470736Z</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 820.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2190.0}</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -2532,7 +2574,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2567,12 +2609,11 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>I don't know. However, I can provide a general approach to identifying such regions:
-- Proximity to major automotive manufacturing hubs
-- Availability of skilled labor force in electronics and manufacturing sectors
-- Presence of established supply chains for raw materials like lithium, cobalt, nickel
-- Government incentives or policies supporting battery production and R&amp;D
-- Access to renewable energy sources for sustainable operations</t>
+          <t>- Southeast Asia: Countries like Thailand, Vietnam, and Indonesia have emerging automotive industries with supportive government policies for electric vehicle (EV) manufacturing.
+- North America: The United States has a robust industrial base and a growing EV market, supported by local supply chains and favorable tax incentives.
+- Europe: Germany and Poland offer established manufacturing ecosystems along with proximity to major car manufacturers and battery suppliers like CATL and LG Energy Solution.
+- China: Despite potential trade barriers, it remains the world's largest EV market with extensive supplier networks and technological advancements in battery technology.
+- South Korea: Home to leading battery companies such as Samsung SDI and LG Chem, providing a strong local supply chain for battery pack assembly.</t>
         </is>
       </c>
       <c r="I15" t="b">
@@ -2581,12 +2622,12 @@
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:31.463702Z</t>
+          <t>2026-03-23T18:21:11.035835Z</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1500.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2560.0}</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -2597,7 +2638,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>20260322T202049Z_qwen14b_no_rag</t>
+          <t>20260323T182038Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2632,10 +2673,11 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>I don't know the specific locations of all emerging electric vehicle (EV) manufacturing clusters outside of major metropolitan areas with absolute certainty. However, based on general trends and reports, here are a few regions where such activity might be occurring:
-- Southeast Asia: Countries like Thailand and Indonesia have been developing their EV industries.
-- Eastern Europe: Some countries in this region are beginning to establish or expand EV production facilities.
-- Latin America: Certain nations in South America are showing interest in building up their EV manufacturing capabilities.</t>
+          <t>- Rural areas in China are seeing the growth of electric vehicle (EV) manufacturing due to government incentives and infrastructure development.
+- Small cities and towns in India are becoming hubs for EV production as local demand increases and startups enter the market.
+- Eastern European countries like Romania and Bulgaria are attracting EV manufacturers with lower operational costs and supportive policies.
+- In North America, smaller cities such as Windsor, Ontario (near Detroit), are leveraging existing automotive industry infrastructure to develop EV manufacturing capabilities.
+- South Korea is expanding its EV production beyond Seoul and Busan, with new plants being established in secondary cities like Daejeon and Gwangju.</t>
         </is>
       </c>
       <c r="I16" t="b">
@@ -2644,12 +2686,12 @@
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-03-22T20:21:33.355808Z</t>
+          <t>2026-03-23T18:21:13.371844Z</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1890.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2340.0}</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>

</xml_diff>

<commit_message>
Qwen no RAG prompt change
</commit_message>
<xml_diff>
--- a/artifacts/response_outputs/qwen14b_no_rag.xlsx
+++ b/artifacts/response_outputs/qwen14b_no_rag.xlsx
@@ -20,13 +20,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,117 +432,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>q_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>question</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>expected_answer</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>resolved_model_name</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>mode</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>prompt_used</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>model_response</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>knowledge_source_data</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>pretrained_data</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>local_context_used</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>web_context_used</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>combined_context_used</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>local_chunk_ids</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>local_chunk_sources</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>local_chunk_texts</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>tavily_chunk_ids</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>tavily_chunk_sources</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>tavily_chunk_texts</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>doc_citations</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>web_citations</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
@@ -539,7 +551,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -575,23 +587,35 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>- Panasonic operates as a Tier 1 supplier for Tesla's EV battery packs, though its primary U.S. facility is in Nevada rather than Georgia or Alabama.
-- SK Innovation (now known as SK On) has significant operations in Georgia with a large battery plant near Atlanta, making it a key Tier 1 supplier for several automakers including Ford and Volkswagen.
-- Samsung SDI operates a Tier 1 EV battery manufacturing facility in Birmingham, Alabama, supplying batteries to various automotive companies.
-- LG Energy Solution is another major player as a Tier 1 supplier but its U.S. operations are primarily located in Michigan rather than Georgia or Alabama.
-- POSCO Chemical, a subsidiary of POSCO Group, acts as a Tier 2 supplier providing battery materials for SK On and other manufacturers with facilities potentially supporting their parent company’s activities in the Southeastern U.S.
-- CATL (Contemporary Amperex Technology Ltd.), while expanding globally, currently does not have direct operations in Georgia or Alabama but supplies through partnerships that may include local suppliers.</t>
+          <t>- **Tier 1 Suppliers**: These are companies that directly supply components to the manufacturers of electric vehicle (EV) battery packs. Examples include:
+  - **Samsung SDI** (illustrative example, not GA/AL-specific): Known for supplying lithium-ion batteries.
+  - **LG Energy Solution** (illustrative example, not GA/AL-specific): A major supplier of EV battery cells.
+- **Tier 2 Suppliers**: These companies supply materials and components to the Tier 1 suppliers. Examples include:
+  - **Umicore** (illustrative example, not GA/AL-specific): Specializes in cathode active materials for lithium-ion batteries.
+  - **Solvay** (illustrative example, not GA/AL-specific): Provides electrolytes and other battery components.
+- **Tier 1/Tier 2 Supplier Types**: 
+  - Tier 1: Battery cell manufacturers, assembly companies.
+  - Tier 2: Material suppliers, component manufacturers.
+- **Illustrative Examples of Potential Suppliers in Georgia and Alabama**:
+  - **Georgia-based Company X** (hypothetical): A local supplier focusing on battery materials.
+  - **Alabama-based Company Y** (hypothetical): Specializes in battery assembly components.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>- Panasonic operates as a Tier 1 supplier for Tesla's EV battery packs, though its primary U.S. facility is in Nevada rather than Georgia or Alabama.
-- SK Innovation (now known as SK On) has significant operations in Georgia with a large battery plant near Atlanta, making it a key Tier 1 supplier for several automakers including Ford and Volkswagen.
-- Samsung SDI operates a Tier 1 EV battery manufacturing facility in Birmingham, Alabama, supplying batteries to various automotive companies.
-- LG Energy Solution is another major player as a Tier 1 supplier but its U.S. operations are primarily located in Michigan rather than Georgia or Alabama.
-- POSCO Chemical, a subsidiary of POSCO Group, acts as a Tier 2 supplier providing battery materials for SK On and other manufacturers with facilities potentially supporting their parent company’s activities in the Southeastern U.S.
-- CATL (Contemporary Amperex Technology Ltd.), while expanding globally, currently does not have direct operations in Georgia or Alabama but supplies through partnerships that may include local suppliers.</t>
+          <t>- **Tier 1 Suppliers**: These are companies that directly supply components to the manufacturers of electric vehicle (EV) battery packs. Examples include:
+  - **Samsung SDI** (illustrative example, not GA/AL-specific): Known for supplying lithium-ion batteries.
+  - **LG Energy Solution** (illustrative example, not GA/AL-specific): A major supplier of EV battery cells.
+- **Tier 2 Suppliers**: These companies supply materials and components to the Tier 1 suppliers. Examples include:
+  - **Umicore** (illustrative example, not GA/AL-specific): Specializes in cathode active materials for lithium-ion batteries.
+  - **Solvay** (illustrative example, not GA/AL-specific): Provides electrolytes and other battery components.
+- **Tier 1/Tier 2 Supplier Types**: 
+  - Tier 1: Battery cell manufacturers, assembly companies.
+  - Tier 2: Material suppliers, component manufacturers.
+- **Illustrative Examples of Potential Suppliers in Georgia and Alabama**:
+  - **Georgia-based Company X** (hypothetical): A local supplier focusing on battery materials.
+  - **Alabama-based Company Y** (hypothetical): Specializes in battery assembly components.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -607,14 +631,14 @@
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:42.453143Z</t>
+          <t>2026-03-23T18:46:42.278301Z</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -650,21 +674,29 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>- Cree Wolfspeed (North Carolina) - Known for silicon carbide semiconductors used in electric vehicle inverters.
-- Infineon Technologies (Georgia Operations) - Produces a range of power electronics components suitable for BEV applications.
-- ON Semiconductor (Tennessee Operations) - Engages in manufacturing power management ICs and discrete devices relevant to BEVs.
-- Texas Instruments (Texas, near Southeast) - Offers motor driver ICs and other power electronics used in electric vehicles.
-- STMicroelectronics (Georgia Operations) - Provides a variety of power modules and IGBTs for automotive applications.</t>
+          <t>- **Tier 1 Suppliers**: These are major companies that produce high-value components directly used by automakers. For power electronics in BEVs, these would include companies like ABB, Siemens Energy, and Hitachi.
+- **Tier 2 Suppliers**: These provide critical subcomponents to Tier 1 suppliers or directly to automakers for integration into the vehicle’s electrical system. Examples might be Infineon Technologies, STMicroelectronics, and Texas Instruments.
+- **Southeastern Locations**: The Southeast U.S. is home to several automotive supplier hubs due to its proximity to major manufacturing centers like Tennessee (Nissan), Alabama (Ford), and Georgia (Stellantis). Key locations for power electronics suppliers might include Atlanta, Nashville, and Birmingham.
+- **Illustrative Examples**:
+  - ABB in Raleigh, North Carolina
+  - Infineon Technologies in Austin, Texas
+  - STMicroelectronics in Dallas, Texas
+- **Partnerships**: Suppliers often partner with local universities or research institutions for innovation. For example, Siemens Energy might collaborate with Georgia Tech on advanced power electronics development.
+- **Regional Clusters**: The Southeastern U.S. has a growing cluster of automotive suppliers and technology firms focusing on electric vehicle components, supported by state incentives and infrastructure investments.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>- Cree Wolfspeed (North Carolina) - Known for silicon carbide semiconductors used in electric vehicle inverters.
-- Infineon Technologies (Georgia Operations) - Produces a range of power electronics components suitable for BEV applications.
-- ON Semiconductor (Tennessee Operations) - Engages in manufacturing power management ICs and discrete devices relevant to BEVs.
-- Texas Instruments (Texas, near Southeast) - Offers motor driver ICs and other power electronics used in electric vehicles.
-- STMicroelectronics (Georgia Operations) - Provides a variety of power modules and IGBTs for automotive applications.</t>
+          <t>- **Tier 1 Suppliers**: These are major companies that produce high-value components directly used by automakers. For power electronics in BEVs, these would include companies like ABB, Siemens Energy, and Hitachi.
+- **Tier 2 Suppliers**: These provide critical subcomponents to Tier 1 suppliers or directly to automakers for integration into the vehicle’s electrical system. Examples might be Infineon Technologies, STMicroelectronics, and Texas Instruments.
+- **Southeastern Locations**: The Southeast U.S. is home to several automotive supplier hubs due to its proximity to major manufacturing centers like Tennessee (Nissan), Alabama (Ford), and Georgia (Stellantis). Key locations for power electronics suppliers might include Atlanta, Nashville, and Birmingham.
+- **Illustrative Examples**:
+  - ABB in Raleigh, North Carolina
+  - Infineon Technologies in Austin, Texas
+  - STMicroelectronics in Dallas, Texas
+- **Partnerships**: Suppliers often partner with local universities or research institutions for innovation. For example, Siemens Energy might collaborate with Georgia Tech on advanced power electronics development.
+- **Regional Clusters**: The Southeastern U.S. has a growing cluster of automotive suppliers and technology firms focusing on electric vehicle components, supported by state incentives and infrastructure investments.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -680,14 +712,14 @@
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:44.690618Z</t>
+          <t>2026-03-23T18:46:46.797032Z</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -723,19 +755,31 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>- Panasonic manufactures battery modules for Tesla at its Nevada Gigafactory.
-- LG Energy Solution produces both battery modules and complete packs for various automakers, including General Motors and Hyundai-Kia.
-- CATL (Contemporary Amperex Technology Ltd) specializes in manufacturing complete battery packs but also supplies modules to companies like Volkswagen.
-- Samsung SDI is known for producing battery modules that are assembled into packs by automotive manufacturers such as BMW and Renault-Nissan-Mitsubishi alliance.</t>
+          <t>- **Tier 1 Companies (Battery Module Manufacturers):** These companies specialize in producing individual battery modules, which are then often assembled into larger battery packs by other manufacturers. Examples include:
+  - Contemporary Amperex Technology (CATL) – known for manufacturing battery modules that can be integrated into various electric vehicle models.
+  - LG Energy Solution – produces a variety of lithium-ion battery modules used in automotive and stationary energy storage applications.
+- **Tier 2 Companies (Battery Pack Assemblers):** These companies typically take the individual battery modules from Tier 1 suppliers and integrate them to form complete battery packs. Examples include:
+  - Panasonic Automotive Systems Company – integrates battery modules into full battery packs for electric vehicles.
+  - Samsung SDI – assembles battery packs using modules supplied by their own manufacturing units or other suppliers.
+- **Regional Focus:** The specific companies mentioned above operate globally but have significant operations in regions like Asia, Europe, and North America. For a more localized perspective, consider regional players such as:
+  - Kokam (South Korea) – specializes in lithium-ion battery packs for electric vehicles.
+  - A123 Systems (United States) – focuses on advanced battery systems including modules and packs.
+- **Illustrative Examples:** Companies like BYD (China), which operates both in manufacturing battery modules and assembling complete battery packs, illustrate the overlap that can exist within a single company.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>- Panasonic manufactures battery modules for Tesla at its Nevada Gigafactory.
-- LG Energy Solution produces both battery modules and complete packs for various automakers, including General Motors and Hyundai-Kia.
-- CATL (Contemporary Amperex Technology Ltd) specializes in manufacturing complete battery packs but also supplies modules to companies like Volkswagen.
-- Samsung SDI is known for producing battery modules that are assembled into packs by automotive manufacturers such as BMW and Renault-Nissan-Mitsubishi alliance.</t>
+          <t>- **Tier 1 Companies (Battery Module Manufacturers):** These companies specialize in producing individual battery modules, which are then often assembled into larger battery packs by other manufacturers. Examples include:
+  - Contemporary Amperex Technology (CATL) – known for manufacturing battery modules that can be integrated into various electric vehicle models.
+  - LG Energy Solution – produces a variety of lithium-ion battery modules used in automotive and stationary energy storage applications.
+- **Tier 2 Companies (Battery Pack Assemblers):** These companies typically take the individual battery modules from Tier 1 suppliers and integrate them to form complete battery packs. Examples include:
+  - Panasonic Automotive Systems Company – integrates battery modules into full battery packs for electric vehicles.
+  - Samsung SDI – assembles battery packs using modules supplied by their own manufacturing units or other suppliers.
+- **Regional Focus:** The specific companies mentioned above operate globally but have significant operations in regions like Asia, Europe, and North America. For a more localized perspective, consider regional players such as:
+  - Kokam (South Korea) – specializes in lithium-ion battery packs for electric vehicles.
+  - A123 Systems (United States) – focuses on advanced battery systems including modules and packs.
+- **Illustrative Examples:** Companies like BYD (China), which operates both in manufacturing battery modules and assembling complete battery packs, illustrate the overlap that can exist within a single company.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -751,14 +795,14 @@
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:46.463003Z</t>
+          <t>2026-03-23T18:46:51.756007Z</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -794,23 +838,43 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>- TE Connectivity in Harrisburg, Texas
-- Molex (a Littelfuse company) with facilities in Irving, Texas
-- Sumitomo Electric Industries with a U.S. base in Plymouth Township, Michigan (near Southeast region)
-- Amphenol Corporation with operations in Atlanta, Georgia
-- Delphi Technologies (now part of Aptiv) has a presence in Troy, Michigan (Southeast proximity)
-- Fujikura Ltd., which operates in Novi, Michigan (close to the Southeast automotive industry hub)</t>
+          <t>- **Tier 1 Suppliers**: Major companies with extensive production capabilities and established presence in the automotive industry.
+  - Illustrative Examples:
+    - TE Connectivity (global, but has significant operations in the Southeast)
+    - Molex (has facilities that could be relevant)
+- **Tier 2 Suppliers**: Smaller companies or divisions of larger corporations specializing in specific components like high-voltage connectors.
+  - Illustrative Examples:
+    - Amphenol Corporation (divisions focusing on automotive electronics)
+    - JAE Electronics (with potential Southeastern manufacturing capabilities)
+- **Regional Manufacturing Firms**: Localized suppliers with specialized expertise and smaller-scale operations but capable of scaling up for automotive production.
+  - Illustrative Examples:
+    - Southern Connector Group (hypothetical example, illustrative only)
+    - Southeast Automotive Connectors Inc. (hypothetical example, illustrative only)
+- **Research Institutions and Universities**: Collaborations or partnerships with research institutions that focus on advanced manufacturing technologies.
+  - Example: Georgia Institute of Technology’s Manufacturing Institute
+- **Government Incentives and Programs**: Utilizing government programs aimed at supporting high-tech manufacturing in the Southeast.
+  - Example: South Carolina Research Authority (SCRA)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>- TE Connectivity in Harrisburg, Texas
-- Molex (a Littelfuse company) with facilities in Irving, Texas
-- Sumitomo Electric Industries with a U.S. base in Plymouth Township, Michigan (near Southeast region)
-- Amphenol Corporation with operations in Atlanta, Georgia
-- Delphi Technologies (now part of Aptiv) has a presence in Troy, Michigan (Southeast proximity)
-- Fujikura Ltd., which operates in Novi, Michigan (close to the Southeast automotive industry hub)</t>
+          <t>- **Tier 1 Suppliers**: Major companies with extensive production capabilities and established presence in the automotive industry.
+  - Illustrative Examples:
+    - TE Connectivity (global, but has significant operations in the Southeast)
+    - Molex (has facilities that could be relevant)
+- **Tier 2 Suppliers**: Smaller companies or divisions of larger corporations specializing in specific components like high-voltage connectors.
+  - Illustrative Examples:
+    - Amphenol Corporation (divisions focusing on automotive electronics)
+    - JAE Electronics (with potential Southeastern manufacturing capabilities)
+- **Regional Manufacturing Firms**: Localized suppliers with specialized expertise and smaller-scale operations but capable of scaling up for automotive production.
+  - Illustrative Examples:
+    - Southern Connector Group (hypothetical example, illustrative only)
+    - Southeast Automotive Connectors Inc. (hypothetical example, illustrative only)
+- **Research Institutions and Universities**: Collaborations or partnerships with research institutions that focus on advanced manufacturing technologies.
+  - Example: Georgia Institute of Technology’s Manufacturing Institute
+- **Government Incentives and Programs**: Utilizing government programs aimed at supporting high-tech manufacturing in the Southeast.
+  - Example: South Carolina Research Authority (SCRA)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -826,14 +890,14 @@
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:48.444272Z</t>
+          <t>2026-03-23T18:46:56.074714Z</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -869,21 +933,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>- ABB Ltd manufactures DC fast charging stations and has contracts with various automakers like BMW, Volkswagen, and Daimler.
-- ChargePoint is a major supplier of EV charging solutions including DC fast chargers and works closely with Ford and other car manufacturers.
-- Eaton Corporation supplies high-power DC charging systems and collaborates with OEMs such as General Motors for fleet vehicles.
-- Schneider Electric produces robust DC fast charging hardware and has partnerships with Renault-Nissan-Mitsubishi Alliance.
-- Siemens Energy offers scalable EV charging solutions, including DC fast chargers, and partners with multiple automakers globally.</t>
+          <t>- ABB Ltd is known for manufacturing DC fast charging stations and has partnerships with various Original Equipment Manufacturers (OEMs).
+- ChargePoint, Inc. provides DC fast charging solutions and collaborates with multiple automakers.
+- Schneider Electric produces EV charging infrastructure and works with several automotive companies.
+- Tier 1 suppliers typically manufacture high-volume components or systems directly for OEMs.
+- Tier 2 suppliers often provide critical subcomponents to the Tier 1 suppliers.
+Illustrative examples (may not be GA/AL-specific):
+- Tier 1: ABB Ltd, ChargePoint Inc., Schneider Electric
+- Tier 2: Example companies might include those specializing in power electronics or battery management systems.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>- ABB Ltd manufactures DC fast charging stations and has contracts with various automakers like BMW, Volkswagen, and Daimler.
-- ChargePoint is a major supplier of EV charging solutions including DC fast chargers and works closely with Ford and other car manufacturers.
-- Eaton Corporation supplies high-power DC charging systems and collaborates with OEMs such as General Motors for fleet vehicles.
-- Schneider Electric produces robust DC fast charging hardware and has partnerships with Renault-Nissan-Mitsubishi Alliance.
-- Siemens Energy offers scalable EV charging solutions, including DC fast chargers, and partners with multiple automakers globally.</t>
+          <t>- ABB Ltd is known for manufacturing DC fast charging stations and has partnerships with various Original Equipment Manufacturers (OEMs).
+- ChargePoint, Inc. provides DC fast charging solutions and collaborates with multiple automakers.
+- Schneider Electric produces EV charging infrastructure and works with several automotive companies.
+- Tier 1 suppliers typically manufacture high-volume components or systems directly for OEMs.
+- Tier 2 suppliers often provide critical subcomponents to the Tier 1 suppliers.
+Illustrative examples (may not be GA/AL-specific):
+- Tier 1: ABB Ltd, ChargePoint Inc., Schneider Electric
+- Tier 2: Example companies might include those specializing in power electronics or battery management systems.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -899,14 +969,14 @@
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:50.625934Z</t>
+          <t>2026-03-23T18:46:58.590394Z</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -942,21 +1012,23 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>- BOSCH: Supplies radar and lidar sensors for autonomous driving.
-- Aptiv (formerly Delphi): Provides advanced driver assistance system components including radar and camera-based solutions.
-- Continental AG: Develops a range of ADAS and autonomous driving sensors, including radar and cameras.
-- Veoneer: Offers sensor fusion systems combining data from multiple types of sensors like radars and cameras.
-- Denso Corporation: Engages in the development of various automotive electronics, including advanced sensing technologies.</t>
+          <t>- **Tier 2 Suppliers for Autonomous Vehicle Sensor Systems**:
+  - **Bosch**: Known for manufacturing a wide range of sensors including radar and lidar, which are crucial for autonomous driving.
+  - **Continental AG**: Provides advanced driver assistance systems (ADAS) that include various sensor technologies such as cameras, radar, and ultrasonic sensors.
+  - **Delphi Technologies**: Offers a variety of sensor solutions including camera-based ADAS and radar systems.
+  - **Veoneer**: Formerly part of Autoliv, Veoneer specializes in advanced safety systems including lidar and radar technology for autonomous vehicles.
+  - **Denso Corporation**: Known for developing various types of sensors used in autonomous driving technologies, such as cameras and radar units.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>- BOSCH: Supplies radar and lidar sensors for autonomous driving.
-- Aptiv (formerly Delphi): Provides advanced driver assistance system components including radar and camera-based solutions.
-- Continental AG: Develops a range of ADAS and autonomous driving sensors, including radar and cameras.
-- Veoneer: Offers sensor fusion systems combining data from multiple types of sensors like radars and cameras.
-- Denso Corporation: Engages in the development of various automotive electronics, including advanced sensing technologies.</t>
+          <t>- **Tier 2 Suppliers for Autonomous Vehicle Sensor Systems**:
+  - **Bosch**: Known for manufacturing a wide range of sensors including radar and lidar, which are crucial for autonomous driving.
+  - **Continental AG**: Provides advanced driver assistance systems (ADAS) that include various sensor technologies such as cameras, radar, and ultrasonic sensors.
+  - **Delphi Technologies**: Offers a variety of sensor solutions including camera-based ADAS and radar systems.
+  - **Veoneer**: Formerly part of Autoliv, Veoneer specializes in advanced safety systems including lidar and radar technology for autonomous vehicles.
+  - **Denso Corporation**: Known for developing various types of sensors used in autonomous driving technologies, such as cameras and radar units.</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
@@ -972,14 +1044,14 @@
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:52.484120Z</t>
+          <t>2026-03-23T18:47:01.422277Z</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1015,21 +1087,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>- Battery cells and modules have high supplier concentration risks due to limited production facilities in the region.
-- Electric motors face similar challenges, with few manufacturers specializing in their production.
-- Power electronics and management systems also exhibit significant supply chain risks because of a lack of local suppliers.
-- Rare earth materials used in EV components are at risk due to reliance on imports from China.
-- Lithium-ion battery raw materials present high concentration risks owing to limited regional sourcing options.</t>
+          <t>- Battery cells and modules often exhibit high supplier concentration due to limited manufacturing capacity globally, which is also true for the Southeast region of the United States.
+- Electric motors and power electronics may have concentrated supply chains if a few dominant manufacturers control production.
+- Rare earth metals used in EV components are typically sourced from a small number of global suppliers, increasing risk.
+- Lithium-ion battery raw materials (e.g., lithium, cobalt) often come from limited geographical sources, creating concentration risks.
+- Charging infrastructure components might face supply chain risks if major charging network providers dominate the Southeast market.
+Illustrative examples:
+- Tier 1: Battery cell manufacturers like Panasonic or LG Energy Solution
+- Tier 2: Rare earth metal suppliers such as Molycorp (USA)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>- Battery cells and modules have high supplier concentration risks due to limited production facilities in the region.
-- Electric motors face similar challenges, with few manufacturers specializing in their production.
-- Power electronics and management systems also exhibit significant supply chain risks because of a lack of local suppliers.
-- Rare earth materials used in EV components are at risk due to reliance on imports from China.
-- Lithium-ion battery raw materials present high concentration risks owing to limited regional sourcing options.</t>
+          <t>- Battery cells and modules often exhibit high supplier concentration due to limited manufacturing capacity globally, which is also true for the Southeast region of the United States.
+- Electric motors and power electronics may have concentrated supply chains if a few dominant manufacturers control production.
+- Rare earth metals used in EV components are typically sourced from a small number of global suppliers, increasing risk.
+- Lithium-ion battery raw materials (e.g., lithium, cobalt) often come from limited geographical sources, creating concentration risks.
+- Charging infrastructure components might face supply chain risks if major charging network providers dominate the Southeast market.
+Illustrative examples:
+- Tier 1: Battery cell manufacturers like Panasonic or LG Energy Solution
+- Tier 2: Rare earth metal suppliers such as Molycorp (USA)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -1045,14 +1123,14 @@
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:54.202886Z</t>
+          <t>2026-03-23T18:47:04.189278Z</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1088,23 +1166,25 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>- Many electric vehicle (EV) manufacturers rely heavily on imported lithium from countries like Chile, Australia, and China for battery production.
-- Cobalt, another critical component in batteries, is predominantly sourced from the Democratic Republic of Congo due to its rich deposits.
-- Supply chain disruptions in these regions can significantly impact battery manufacturing capacity globally.
-- The geopolitical tensions between major importing nations and exporting countries affect supply stability and pricing.
-- Diversification efforts are underway by companies to secure alternative sources and reduce dependency on single-country imports.
-- Recycling initiatives for spent batteries aim to create a more sustainable and less dependent supply chain in the long term.</t>
+          <t>- **Raw Material Imports**: Many countries rely heavily on imported raw materials such as lithium, cobalt, and nickel from countries like Chile, Congo, and Indonesia for battery production.
+- **Manufacturing Components**: Battery manufacturing often requires specialized components that may be sourced internationally due to technological or logistical advantages in certain regions.
+- **Technological Dependencies**: Advanced technologies used in battery production might come from leading technology hubs such as South Korea (LG Chem) or Japan (Panasonic), which can influence supply chain dynamics.
+- **Logistical Challenges**: International shipping and logistics play a critical role, with potential disruptions due to geopolitical tensions, natural disasters, or pandemics affecting global trade routes.
+- **Regulatory Compliance**: Adherence to international regulations and standards is crucial for battery manufacturers, impacting sourcing decisions and operational costs.
+- **Tier 1 Suppliers**: Major players like China’s CATL (Contemporary Amperex Technology Ltd) and South Korea’s Samsung SDI are key suppliers in the global battery market.
+- **Tier 2 Suppliers**: Smaller but significant suppliers include companies that specialize in specific materials or components, such as Albemarle Corporation for lithium processing.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>- Many electric vehicle (EV) manufacturers rely heavily on imported lithium from countries like Chile, Australia, and China for battery production.
-- Cobalt, another critical component in batteries, is predominantly sourced from the Democratic Republic of Congo due to its rich deposits.
-- Supply chain disruptions in these regions can significantly impact battery manufacturing capacity globally.
-- The geopolitical tensions between major importing nations and exporting countries affect supply stability and pricing.
-- Diversification efforts are underway by companies to secure alternative sources and reduce dependency on single-country imports.
-- Recycling initiatives for spent batteries aim to create a more sustainable and less dependent supply chain in the long term.</t>
+          <t>- **Raw Material Imports**: Many countries rely heavily on imported raw materials such as lithium, cobalt, and nickel from countries like Chile, Congo, and Indonesia for battery production.
+- **Manufacturing Components**: Battery manufacturing often requires specialized components that may be sourced internationally due to technological or logistical advantages in certain regions.
+- **Technological Dependencies**: Advanced technologies used in battery production might come from leading technology hubs such as South Korea (LG Chem) or Japan (Panasonic), which can influence supply chain dynamics.
+- **Logistical Challenges**: International shipping and logistics play a critical role, with potential disruptions due to geopolitical tensions, natural disasters, or pandemics affecting global trade routes.
+- **Regulatory Compliance**: Adherence to international regulations and standards is crucial for battery manufacturers, impacting sourcing decisions and operational costs.
+- **Tier 1 Suppliers**: Major players like China’s CATL (Contemporary Amperex Technology Ltd) and South Korea’s Samsung SDI are key suppliers in the global battery market.
+- **Tier 2 Suppliers**: Smaller but significant suppliers include companies that specialize in specific materials or components, such as Albemarle Corporation for lithium processing.</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -1120,14 +1200,14 @@
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:56.503286Z</t>
+          <t>2026-03-23T18:47:08.343936Z</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1163,23 +1243,29 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>- Tier 2 and Tier 3 bottlenecks can significantly affect the supply chain efficiency of Original Equipment Manufacturers (OEMs).
-- Delays in obtaining components from Tier 2 suppliers can lead to reduced output at assembly lines, impacting overall production schedules.
-- Quality issues with Tier 3 parts can cascade up through the supply chain, causing rework and delays for OEMs.
-- Shortages or disruptions in raw materials supplied by Tier 3 vendors can limit the availability of critical components needed by Tier 2 suppliers.
-- Inflexible logistics from Tier 2 and Tier 3 suppliers can cause bottlenecks in inventory management at OEM facilities.
-- Communication breakdowns between lower-tier suppliers and OEMs can result in mismatches in production forecasts, leading to excess or shortage issues.</t>
+          <t>- **Supply Chain Disruptions:** Tier 2 and Tier 3 suppliers often have less robust supply chains, leading to potential disruptions that can affect the availability of critical components for OEMs.
+- **Quality Control Issues:** Smaller suppliers may lack advanced quality control measures, resulting in defective parts that delay production lines at OEM facilities.
+- **Capacity Constraints:** Limited manufacturing capacity at Tier 2 and Tier 3 vendors can cause bottlenecks when there is unexpected demand or sudden increases in orders from OEMs.
+- **Technological Limitations:** Smaller suppliers might not have the latest technology, leading to slower production times and inefficiencies that impact OEM schedules.
+- **Financial Instability:** Financial difficulties at lower-tier suppliers can lead to delayed deliveries or even bankruptcy, causing significant disruptions for OEMs.
+- **Logistical Challenges:** Tier 2 and Tier 3 companies often face logistical challenges such as transportation delays or storage issues, which can impede the timely delivery of parts to OEM production lines.
+Illustrative examples:
+- A small electronics manufacturer (Tier 3) facing a sudden shortage of raw materials due to global supply chain disruptions.
+- A medium-sized supplier (Tier 2) experiencing quality control failures that require extensive rework and delays in part deliveries.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>- Tier 2 and Tier 3 bottlenecks can significantly affect the supply chain efficiency of Original Equipment Manufacturers (OEMs).
-- Delays in obtaining components from Tier 2 suppliers can lead to reduced output at assembly lines, impacting overall production schedules.
-- Quality issues with Tier 3 parts can cascade up through the supply chain, causing rework and delays for OEMs.
-- Shortages or disruptions in raw materials supplied by Tier 3 vendors can limit the availability of critical components needed by Tier 2 suppliers.
-- Inflexible logistics from Tier 2 and Tier 3 suppliers can cause bottlenecks in inventory management at OEM facilities.
-- Communication breakdowns between lower-tier suppliers and OEMs can result in mismatches in production forecasts, leading to excess or shortage issues.</t>
+          <t>- **Supply Chain Disruptions:** Tier 2 and Tier 3 suppliers often have less robust supply chains, leading to potential disruptions that can affect the availability of critical components for OEMs.
+- **Quality Control Issues:** Smaller suppliers may lack advanced quality control measures, resulting in defective parts that delay production lines at OEM facilities.
+- **Capacity Constraints:** Limited manufacturing capacity at Tier 2 and Tier 3 vendors can cause bottlenecks when there is unexpected demand or sudden increases in orders from OEMs.
+- **Technological Limitations:** Smaller suppliers might not have the latest technology, leading to slower production times and inefficiencies that impact OEM schedules.
+- **Financial Instability:** Financial difficulties at lower-tier suppliers can lead to delayed deliveries or even bankruptcy, causing significant disruptions for OEMs.
+- **Logistical Challenges:** Tier 2 and Tier 3 companies often face logistical challenges such as transportation delays or storage issues, which can impede the timely delivery of parts to OEM production lines.
+Illustrative examples:
+- A small electronics manufacturer (Tier 3) facing a sudden shortage of raw materials due to global supply chain disruptions.
+- A medium-sized supplier (Tier 2) experiencing quality control failures that require extensive rework and delays in part deliveries.</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -1195,14 +1281,14 @@
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:59.393016Z</t>
+          <t>2026-03-23T18:47:12.893271Z</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1238,21 +1324,23 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>- Battery manufacturing and recycling facilities are expanding rapidly due to proximity to automotive assembly plants.
-- Charging infrastructure installation companies are seeing significant growth as electric vehicle adoption increases.
-- Lithium-ion battery component suppliers are establishing regional hubs for quicker delivery times.
-- Electric vehicle (EV) service centers specializing in EV maintenance and repair are proliferating.
-- Regional distribution networks for EV parts and components are becoming more efficient and extensive.</t>
+          <t>- Battery manufacturing and recycling facilities are expanding rapidly due to increased demand for electric vehicles (EVs).
+- Charging infrastructure installation companies are seeing significant growth as more public charging stations are required to support EV adoption.
+- Lithium-ion battery component suppliers are experiencing strong growth, driven by the need for advanced materials in EV batteries.
+- Electric vehicle assembly plants are being established or expanded by major automakers looking to capitalize on regional incentives and supply chain proximity.
+- Tier 1 illustrative examples: Battery manufacturing (e.g., LG Energy Solution), Charging infrastructure providers (e.g., ChargePoint).
+- Tier 2 illustrative examples: Component suppliers for battery materials, Local charging station installation companies.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>- Battery manufacturing and recycling facilities are expanding rapidly due to proximity to automotive assembly plants.
-- Charging infrastructure installation companies are seeing significant growth as electric vehicle adoption increases.
-- Lithium-ion battery component suppliers are establishing regional hubs for quicker delivery times.
-- Electric vehicle (EV) service centers specializing in EV maintenance and repair are proliferating.
-- Regional distribution networks for EV parts and components are becoming more efficient and extensive.</t>
+          <t>- Battery manufacturing and recycling facilities are expanding rapidly due to increased demand for electric vehicles (EVs).
+- Charging infrastructure installation companies are seeing significant growth as more public charging stations are required to support EV adoption.
+- Lithium-ion battery component suppliers are experiencing strong growth, driven by the need for advanced materials in EV batteries.
+- Electric vehicle assembly plants are being established or expanded by major automakers looking to capitalize on regional incentives and supply chain proximity.
+- Tier 1 illustrative examples: Battery manufacturing (e.g., LG Energy Solution), Charging infrastructure providers (e.g., ChargePoint).
+- Tier 2 illustrative examples: Component suppliers for battery materials, Local charging station installation companies.</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -1268,14 +1356,14 @@
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:00.957549Z</t>
+          <t>2026-03-23T18:47:15.401453Z</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1311,21 +1399,21 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>- Volkswagen has committed significant resources to electric vehicle production and is phasing out traditional internal combustion engine (ICE) vehicles in many markets.
-- General Motors is investing heavily in battery technology and plans to launch multiple new electric models, reducing focus on conventional engines.
-- Ford Motor Company is expanding its EV lineup with the Mustang Mach-E and F-150 Lightning while scaling back some ICE vehicle production lines.
-- Toyota has announced a shift towards hybrid and fully electric vehicles as part of its long-term strategy, though it continues to support traditional ICE technology in certain markets.
-- Hyundai-Kia is rapidly growing its portfolio of electric cars and plans substantial investments in battery manufacturing facilities.</t>
+          <t>- Automotive giants like General Motors and Volkswagen are transitioning their product lines towards electric vehicles (EVs), phasing out internal combustion engine (ICE) components.
+- Suppliers such as Bosch and Continental are adapting by developing new technologies for EVs, including battery management systems and electric drivetrains.
+- Startups focused on EV technology, such as Rivian and Lucid Motors, are gaining traction and influencing established companies to shift their focus towards EV products.
+- Traditional ICE component manufacturers like Delphi Technologies are rebranding and restructuring to emphasize their role in the EV supply chain.
+- Companies like Panasonic, which have a strong presence in battery manufacturing for consumer electronics, are expanding into automotive batteries for EVs.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>- Volkswagen has committed significant resources to electric vehicle production and is phasing out traditional internal combustion engine (ICE) vehicles in many markets.
-- General Motors is investing heavily in battery technology and plans to launch multiple new electric models, reducing focus on conventional engines.
-- Ford Motor Company is expanding its EV lineup with the Mustang Mach-E and F-150 Lightning while scaling back some ICE vehicle production lines.
-- Toyota has announced a shift towards hybrid and fully electric vehicles as part of its long-term strategy, though it continues to support traditional ICE technology in certain markets.
-- Hyundai-Kia is rapidly growing its portfolio of electric cars and plans substantial investments in battery manufacturing facilities.</t>
+          <t>- Automotive giants like General Motors and Volkswagen are transitioning their product lines towards electric vehicles (EVs), phasing out internal combustion engine (ICE) components.
+- Suppliers such as Bosch and Continental are adapting by developing new technologies for EVs, including battery management systems and electric drivetrains.
+- Startups focused on EV technology, such as Rivian and Lucid Motors, are gaining traction and influencing established companies to shift their focus towards EV products.
+- Traditional ICE component manufacturers like Delphi Technologies are rebranding and restructuring to emphasize their role in the EV supply chain.
+- Companies like Panasonic, which have a strong presence in battery manufacturing for consumer electronics, are expanding into automotive batteries for EVs.</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
@@ -1341,14 +1429,14 @@
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:03.409028Z</t>
+          <t>2026-03-23T18:47:17.976334Z</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1384,23 +1472,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>- Demand for battery manufacturing equipment is increasing in Asia due to the rapid growth of electric vehicle (EV) markets and government incentives in countries like China and South Korea.
-- Europe is also seeing significant growth, driven by ambitious climate goals and investments from major automakers such as Volkswagen and BMW.
-- North America is experiencing strong demand, particularly in the United States, where there are substantial federal and state-level initiatives to support EV infrastructure and battery production.
-- Latin American countries like Brazil and Chile are showing interest due to their rich lithium reserves and growing automotive industries.
-- In Africa, regions with significant mineral resources are attracting investments for battery manufacturing as global supply chains diversify.
-- Middle Eastern nations are exploring opportunities in battery manufacturing to reduce reliance on oil exports and capitalize on renewable energy initiatives.</t>
+          <t>- Demand for battery manufacturing equipment is increasing in regions with significant investments in electric vehicle (EV) and renewable energy sectors, such as Asia-Pacific, Europe, and North America.
+- China has seen a surge in demand due to government incentives supporting EV production and storage solutions.
+- The European Union is focusing on localizing battery production to reduce reliance on imports and meet ambitious climate goals.
+- In the United States, states like California and Michigan are experiencing high demand as automakers expand their EV manufacturing capabilities.
+- South Korea and Japan are also seeing increased demand due to established electronics and automotive industries investing in advanced battery technologies.
+- Illustrative examples of regions with growing demand include:
+  - Tier 1: Asia-Pacific (China, South Korea)
+  - Tier 2: Europe (Germany, Poland), North America (California, Michigan)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>- Demand for battery manufacturing equipment is increasing in Asia due to the rapid growth of electric vehicle (EV) markets and government incentives in countries like China and South Korea.
-- Europe is also seeing significant growth, driven by ambitious climate goals and investments from major automakers such as Volkswagen and BMW.
-- North America is experiencing strong demand, particularly in the United States, where there are substantial federal and state-level initiatives to support EV infrastructure and battery production.
-- Latin American countries like Brazil and Chile are showing interest due to their rich lithium reserves and growing automotive industries.
-- In Africa, regions with significant mineral resources are attracting investments for battery manufacturing as global supply chains diversify.
-- Middle Eastern nations are exploring opportunities in battery manufacturing to reduce reliance on oil exports and capitalize on renewable energy initiatives.</t>
+          <t>- Demand for battery manufacturing equipment is increasing in regions with significant investments in electric vehicle (EV) and renewable energy sectors, such as Asia-Pacific, Europe, and North America.
+- China has seen a surge in demand due to government incentives supporting EV production and storage solutions.
+- The European Union is focusing on localizing battery production to reduce reliance on imports and meet ambitious climate goals.
+- In the United States, states like California and Michigan are experiencing high demand as automakers expand their EV manufacturing capabilities.
+- South Korea and Japan are also seeing increased demand due to established electronics and automotive industries investing in advanced battery technologies.
+- Illustrative examples of regions with growing demand include:
+  - Tier 1: Asia-Pacific (China, South Korea)
+  - Tier 2: Europe (Germany, Poland), North America (California, Michigan)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -1416,14 +1508,14 @@
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:06.279677Z</t>
+          <t>2026-03-23T18:47:21.001963Z</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1459,21 +1551,25 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>- Miami-Dade County, Florida: High concentration of electric vehicle (EV) suppliers and a large workforce in the automotive industry.
-- Orange County, Florida: Presence of EV charging infrastructure companies and significant employment opportunities in tech and manufacturing sectors.
-- Harris County, Texas: Home to multiple EV component manufacturers and a robust labor market with skilled workers.
-- Maricopa County, Arizona: Growing presence of EV startups and established suppliers, along with a trainable workforce due to local educational institutions.
-- Clark County, Nevada: Increasing number of EV-related businesses and a growing tech-savvy workforce.</t>
+          <t>- Counties in the Southeastern United States that are likely to have high electric vehicle (EV) supplier density and a robust workforce include those near major automotive manufacturing hubs.
+- Illustrative examples of such counties might be:
+  - Shelby County, Alabama: Home to Ford Motor Company’s River Rouge Complex, which has shown interest in EV production.
+  - Greenville County, South Carolina: Known for its strong automotive industry presence, including BMW's plant and numerous suppliers.
+- These areas typically have established infrastructure and a skilled workforce trained in manufacturing processes relevant to EV production.
+- Counties with universities or technical colleges that offer specialized training programs related to automotive engineering and technology are also likely candidates.
+- Tier 1 counties would be those directly adjacent to major automotive plants, while Tier 2 might include nearby counties with significant supplier networks but slightly less direct plant proximity.</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>- Miami-Dade County, Florida: High concentration of electric vehicle (EV) suppliers and a large workforce in the automotive industry.
-- Orange County, Florida: Presence of EV charging infrastructure companies and significant employment opportunities in tech and manufacturing sectors.
-- Harris County, Texas: Home to multiple EV component manufacturers and a robust labor market with skilled workers.
-- Maricopa County, Arizona: Growing presence of EV startups and established suppliers, along with a trainable workforce due to local educational institutions.
-- Clark County, Nevada: Increasing number of EV-related businesses and a growing tech-savvy workforce.</t>
+          <t>- Counties in the Southeastern United States that are likely to have high electric vehicle (EV) supplier density and a robust workforce include those near major automotive manufacturing hubs.
+- Illustrative examples of such counties might be:
+  - Shelby County, Alabama: Home to Ford Motor Company’s River Rouge Complex, which has shown interest in EV production.
+  - Greenville County, South Carolina: Known for its strong automotive industry presence, including BMW's plant and numerous suppliers.
+- These areas typically have established infrastructure and a skilled workforce trained in manufacturing processes relevant to EV production.
+- Counties with universities or technical colleges that offer specialized training programs related to automotive engineering and technology are also likely candidates.
+- Tier 1 counties would be those directly adjacent to major automotive plants, while Tier 2 might include nearby counties with significant supplier networks but slightly less direct plant proximity.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -1489,14 +1585,14 @@
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:08.470736Z</t>
+          <t>2026-03-23T18:47:24.072727Z</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1532,21 +1628,21 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>- Southeast Asia: Countries like Thailand, Vietnam, and Indonesia have emerging automotive industries with supportive government policies for electric vehicle (EV) manufacturing.
-- North America: The United States has a robust industrial base and a growing EV market, supported by local supply chains and favorable tax incentives.
-- Europe: Germany and Poland offer established manufacturing ecosystems along with proximity to major car manufacturers and battery suppliers like CATL and LG Energy Solution.
-- China: Despite potential trade barriers, it remains the world's largest EV market with extensive supplier networks and technological advancements in battery technology.
-- South Korea: Home to leading battery companies such as Samsung SDI and LG Chem, providing a strong local supply chain for battery pack assembly.</t>
+          <t>- **Tier 1 Regions:** Areas with established automotive manufacturing hubs, robust supply chains, and favorable government policies supporting electric vehicle (EV) production.
+- **Tier 2 Regions:** Locations that are emerging in the EV sector but may lack some of the mature infrastructure found in Tier 1 regions.
+**Illustrative Examples:**
+- **Southeastern United States:** Tennessee, with its strong automotive industry presence around Nashville and Memphis, and Alabama, home to major automotive manufacturing facilities.
+- **East Asia:** South Korea’s Ulsan region, known for its concentration of automotive manufacturers and suppliers.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>- Southeast Asia: Countries like Thailand, Vietnam, and Indonesia have emerging automotive industries with supportive government policies for electric vehicle (EV) manufacturing.
-- North America: The United States has a robust industrial base and a growing EV market, supported by local supply chains and favorable tax incentives.
-- Europe: Germany and Poland offer established manufacturing ecosystems along with proximity to major car manufacturers and battery suppliers like CATL and LG Energy Solution.
-- China: Despite potential trade barriers, it remains the world's largest EV market with extensive supplier networks and technological advancements in battery technology.
-- South Korea: Home to leading battery companies such as Samsung SDI and LG Chem, providing a strong local supply chain for battery pack assembly.</t>
+          <t>- **Tier 1 Regions:** Areas with established automotive manufacturing hubs, robust supply chains, and favorable government policies supporting electric vehicle (EV) production.
+- **Tier 2 Regions:** Locations that are emerging in the EV sector but may lack some of the mature infrastructure found in Tier 1 regions.
+**Illustrative Examples:**
+- **Southeastern United States:** Tennessee, with its strong automotive industry presence around Nashville and Memphis, and Alabama, home to major automotive manufacturing facilities.
+- **East Asia:** South Korea’s Ulsan region, known for its concentration of automotive manufacturers and suppliers.</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -1562,14 +1658,14 @@
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:11.035835Z</t>
+          <t>2026-03-23T18:47:26.306040Z</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1605,21 +1701,23 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>- Rural areas in China are seeing the growth of electric vehicle (EV) manufacturing due to government incentives and infrastructure development.
-- Small cities and towns in India are becoming hubs for EV production as local demand increases and startups enter the market.
-- Eastern European countries like Romania and Bulgaria are attracting EV manufacturers with lower operational costs and supportive policies.
-- In North America, smaller cities such as Windsor, Ontario (near Detroit), are leveraging existing automotive industry infrastructure to develop EV manufacturing capabilities.
-- South Korea is expanding its EV production beyond Seoul and Busan, with new plants being established in secondary cities like Daejeon and Gwangju.</t>
+          <t>- Emerging electric vehicle (EV) manufacturing clusters can be found in smaller cities and rural areas that offer lower operational costs, abundant land for factory sites, and supportive local policies. 
+- For example, the U.S. state of Michigan has seen growth in EV manufacturing beyond Detroit, with companies establishing plants in cities like Holland.
+- Another illustrative example is the city of Sunderland in the UK, where Nissan established an EV production facility outside London and other major metropolitan areas.
+- Tier 1 locations would be smaller industrial or suburban towns near existing automotive supply chains but with lower real estate costs. 
+- Tier 2 locations might include rural regions that offer tax incentives for green manufacturing initiatives.
+- These clusters often benefit from government grants, research partnerships with local universities, and a skilled workforce trained in traditional automotive industries.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>- Rural areas in China are seeing the growth of electric vehicle (EV) manufacturing due to government incentives and infrastructure development.
-- Small cities and towns in India are becoming hubs for EV production as local demand increases and startups enter the market.
-- Eastern European countries like Romania and Bulgaria are attracting EV manufacturers with lower operational costs and supportive policies.
-- In North America, smaller cities such as Windsor, Ontario (near Detroit), are leveraging existing automotive industry infrastructure to develop EV manufacturing capabilities.
-- South Korea is expanding its EV production beyond Seoul and Busan, with new plants being established in secondary cities like Daejeon and Gwangju.</t>
+          <t>- Emerging electric vehicle (EV) manufacturing clusters can be found in smaller cities and rural areas that offer lower operational costs, abundant land for factory sites, and supportive local policies. 
+- For example, the U.S. state of Michigan has seen growth in EV manufacturing beyond Detroit, with companies establishing plants in cities like Holland.
+- Another illustrative example is the city of Sunderland in the UK, where Nissan established an EV production facility outside London and other major metropolitan areas.
+- Tier 1 locations would be smaller industrial or suburban towns near existing automotive supply chains but with lower real estate costs. 
+- Tier 2 locations might include rural regions that offer tax incentives for green manufacturing initiatives.
+- These clusters often benefit from government grants, research partnerships with local universities, and a skilled workforce trained in traditional automotive industries.</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
@@ -1635,7 +1733,7 @@
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:13.371844Z</t>
+          <t>2026-03-23T18:47:29.255100Z</t>
         </is>
       </c>
     </row>
@@ -1654,82 +1752,82 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>q_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>question</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>resolved_model_name</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>mode</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>prompt_used</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>answer_text</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>error_message</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>timing</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>tokens_in</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>tokens_out</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>tokens_total</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>cost_usd</t>
         </is>
@@ -1738,7 +1836,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1773,12 +1871,18 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>- Panasonic operates as a Tier 1 supplier for Tesla's EV battery packs, though its primary U.S. facility is in Nevada rather than Georgia or Alabama.
-- SK Innovation (now known as SK On) has significant operations in Georgia with a large battery plant near Atlanta, making it a key Tier 1 supplier for several automakers including Ford and Volkswagen.
-- Samsung SDI operates a Tier 1 EV battery manufacturing facility in Birmingham, Alabama, supplying batteries to various automotive companies.
-- LG Energy Solution is another major player as a Tier 1 supplier but its U.S. operations are primarily located in Michigan rather than Georgia or Alabama.
-- POSCO Chemical, a subsidiary of POSCO Group, acts as a Tier 2 supplier providing battery materials for SK On and other manufacturers with facilities potentially supporting their parent company’s activities in the Southeastern U.S.
-- CATL (Contemporary Amperex Technology Ltd.), while expanding globally, currently does not have direct operations in Georgia or Alabama but supplies through partnerships that may include local suppliers.</t>
+          <t>- **Tier 1 Suppliers**: These are companies that directly supply components to the manufacturers of electric vehicle (EV) battery packs. Examples include:
+  - **Samsung SDI** (illustrative example, not GA/AL-specific): Known for supplying lithium-ion batteries.
+  - **LG Energy Solution** (illustrative example, not GA/AL-specific): A major supplier of EV battery cells.
+- **Tier 2 Suppliers**: These companies supply materials and components to the Tier 1 suppliers. Examples include:
+  - **Umicore** (illustrative example, not GA/AL-specific): Specializes in cathode active materials for lithium-ion batteries.
+  - **Solvay** (illustrative example, not GA/AL-specific): Provides electrolytes and other battery components.
+- **Tier 1/Tier 2 Supplier Types**: 
+  - Tier 1: Battery cell manufacturers, assembly companies.
+  - Tier 2: Material suppliers, component manufacturers.
+- **Illustrative Examples of Potential Suppliers in Georgia and Alabama**:
+  - **Georgia-based Company X** (hypothetical): A local supplier focusing on battery materials.
+  - **Alabama-based Company Y** (hypothetical): Specializes in battery assembly components.</t>
         </is>
       </c>
       <c r="I2" t="b">
@@ -1787,12 +1891,12 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:42.453143Z</t>
+          <t>2026-03-23T18:46:42.278301Z</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 3730.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 7480.0}</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -1803,7 +1907,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1838,11 +1942,15 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>- Cree Wolfspeed (North Carolina) - Known for silicon carbide semiconductors used in electric vehicle inverters.
-- Infineon Technologies (Georgia Operations) - Produces a range of power electronics components suitable for BEV applications.
-- ON Semiconductor (Tennessee Operations) - Engages in manufacturing power management ICs and discrete devices relevant to BEVs.
-- Texas Instruments (Texas, near Southeast) - Offers motor driver ICs and other power electronics used in electric vehicles.
-- STMicroelectronics (Georgia Operations) - Provides a variety of power modules and IGBTs for automotive applications.</t>
+          <t>- **Tier 1 Suppliers**: These are major companies that produce high-value components directly used by automakers. For power electronics in BEVs, these would include companies like ABB, Siemens Energy, and Hitachi.
+- **Tier 2 Suppliers**: These provide critical subcomponents to Tier 1 suppliers or directly to automakers for integration into the vehicle’s electrical system. Examples might be Infineon Technologies, STMicroelectronics, and Texas Instruments.
+- **Southeastern Locations**: The Southeast U.S. is home to several automotive supplier hubs due to its proximity to major manufacturing centers like Tennessee (Nissan), Alabama (Ford), and Georgia (Stellantis). Key locations for power electronics suppliers might include Atlanta, Nashville, and Birmingham.
+- **Illustrative Examples**:
+  - ABB in Raleigh, North Carolina
+  - Infineon Technologies in Austin, Texas
+  - STMicroelectronics in Dallas, Texas
+- **Partnerships**: Suppliers often partner with local universities or research institutions for innovation. For example, Siemens Energy might collaborate with Georgia Tech on advanced power electronics development.
+- **Regional Clusters**: The Southeastern U.S. has a growing cluster of automotive suppliers and technology firms focusing on electric vehicle components, supported by state incentives and infrastructure investments.</t>
         </is>
       </c>
       <c r="I3" t="b">
@@ -1851,12 +1959,12 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:44.690618Z</t>
+          <t>2026-03-23T18:46:46.797032Z</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2240.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 4520.0}</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -1867,7 +1975,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1902,10 +2010,16 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>- Panasonic manufactures battery modules for Tesla at its Nevada Gigafactory.
-- LG Energy Solution produces both battery modules and complete packs for various automakers, including General Motors and Hyundai-Kia.
-- CATL (Contemporary Amperex Technology Ltd) specializes in manufacturing complete battery packs but also supplies modules to companies like Volkswagen.
-- Samsung SDI is known for producing battery modules that are assembled into packs by automotive manufacturers such as BMW and Renault-Nissan-Mitsubishi alliance.</t>
+          <t>- **Tier 1 Companies (Battery Module Manufacturers):** These companies specialize in producing individual battery modules, which are then often assembled into larger battery packs by other manufacturers. Examples include:
+  - Contemporary Amperex Technology (CATL) – known for manufacturing battery modules that can be integrated into various electric vehicle models.
+  - LG Energy Solution – produces a variety of lithium-ion battery modules used in automotive and stationary energy storage applications.
+- **Tier 2 Companies (Battery Pack Assemblers):** These companies typically take the individual battery modules from Tier 1 suppliers and integrate them to form complete battery packs. Examples include:
+  - Panasonic Automotive Systems Company – integrates battery modules into full battery packs for electric vehicles.
+  - Samsung SDI – assembles battery packs using modules supplied by their own manufacturing units or other suppliers.
+- **Regional Focus:** The specific companies mentioned above operate globally but have significant operations in regions like Asia, Europe, and North America. For a more localized perspective, consider regional players such as:
+  - Kokam (South Korea) – specializes in lithium-ion battery packs for electric vehicles.
+  - A123 Systems (United States) – focuses on advanced battery systems including modules and packs.
+- **Illustrative Examples:** Companies like BYD (China), which operates both in manufacturing battery modules and assembling complete battery packs, illustrate the overlap that can exist within a single company.</t>
         </is>
       </c>
       <c r="I4" t="b">
@@ -1914,12 +2028,12 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:46.463003Z</t>
+          <t>2026-03-23T18:46:51.756007Z</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1770.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 4960.0}</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -1930,7 +2044,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1965,12 +2079,22 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>- TE Connectivity in Harrisburg, Texas
-- Molex (a Littelfuse company) with facilities in Irving, Texas
-- Sumitomo Electric Industries with a U.S. base in Plymouth Township, Michigan (near Southeast region)
-- Amphenol Corporation with operations in Atlanta, Georgia
-- Delphi Technologies (now part of Aptiv) has a presence in Troy, Michigan (Southeast proximity)
-- Fujikura Ltd., which operates in Novi, Michigan (close to the Southeast automotive industry hub)</t>
+          <t>- **Tier 1 Suppliers**: Major companies with extensive production capabilities and established presence in the automotive industry.
+  - Illustrative Examples:
+    - TE Connectivity (global, but has significant operations in the Southeast)
+    - Molex (has facilities that could be relevant)
+- **Tier 2 Suppliers**: Smaller companies or divisions of larger corporations specializing in specific components like high-voltage connectors.
+  - Illustrative Examples:
+    - Amphenol Corporation (divisions focusing on automotive electronics)
+    - JAE Electronics (with potential Southeastern manufacturing capabilities)
+- **Regional Manufacturing Firms**: Localized suppliers with specialized expertise and smaller-scale operations but capable of scaling up for automotive production.
+  - Illustrative Examples:
+    - Southern Connector Group (hypothetical example, illustrative only)
+    - Southeast Automotive Connectors Inc. (hypothetical example, illustrative only)
+- **Research Institutions and Universities**: Collaborations or partnerships with research institutions that focus on advanced manufacturing technologies.
+  - Example: Georgia Institute of Technology’s Manufacturing Institute
+- **Government Incentives and Programs**: Utilizing government programs aimed at supporting high-tech manufacturing in the Southeast.
+  - Example: South Carolina Research Authority (SCRA)</t>
         </is>
       </c>
       <c r="I5" t="b">
@@ -1979,12 +2103,12 @@
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:48.444272Z</t>
+          <t>2026-03-23T18:46:56.074714Z</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1980.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 4320.0}</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1995,7 +2119,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2030,11 +2154,14 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>- ABB Ltd manufactures DC fast charging stations and has contracts with various automakers like BMW, Volkswagen, and Daimler.
-- ChargePoint is a major supplier of EV charging solutions including DC fast chargers and works closely with Ford and other car manufacturers.
-- Eaton Corporation supplies high-power DC charging systems and collaborates with OEMs such as General Motors for fleet vehicles.
-- Schneider Electric produces robust DC fast charging hardware and has partnerships with Renault-Nissan-Mitsubishi Alliance.
-- Siemens Energy offers scalable EV charging solutions, including DC fast chargers, and partners with multiple automakers globally.</t>
+          <t>- ABB Ltd is known for manufacturing DC fast charging stations and has partnerships with various Original Equipment Manufacturers (OEMs).
+- ChargePoint, Inc. provides DC fast charging solutions and collaborates with multiple automakers.
+- Schneider Electric produces EV charging infrastructure and works with several automotive companies.
+- Tier 1 suppliers typically manufacture high-volume components or systems directly for OEMs.
+- Tier 2 suppliers often provide critical subcomponents to the Tier 1 suppliers.
+Illustrative examples (may not be GA/AL-specific):
+- Tier 1: ABB Ltd, ChargePoint Inc., Schneider Electric
+- Tier 2: Example companies might include those specializing in power electronics or battery management systems.</t>
         </is>
       </c>
       <c r="I6" t="b">
@@ -2043,12 +2170,12 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:50.625934Z</t>
+          <t>2026-03-23T18:46:58.590394Z</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2180.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2520.0}</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -2059,7 +2186,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2094,11 +2221,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>- BOSCH: Supplies radar and lidar sensors for autonomous driving.
-- Aptiv (formerly Delphi): Provides advanced driver assistance system components including radar and camera-based solutions.
-- Continental AG: Develops a range of ADAS and autonomous driving sensors, including radar and cameras.
-- Veoneer: Offers sensor fusion systems combining data from multiple types of sensors like radars and cameras.
-- Denso Corporation: Engages in the development of various automotive electronics, including advanced sensing technologies.</t>
+          <t>- **Tier 2 Suppliers for Autonomous Vehicle Sensor Systems**:
+  - **Bosch**: Known for manufacturing a wide range of sensors including radar and lidar, which are crucial for autonomous driving.
+  - **Continental AG**: Provides advanced driver assistance systems (ADAS) that include various sensor technologies such as cameras, radar, and ultrasonic sensors.
+  - **Delphi Technologies**: Offers a variety of sensor solutions including camera-based ADAS and radar systems.
+  - **Veoneer**: Formerly part of Autoliv, Veoneer specializes in advanced safety systems including lidar and radar technology for autonomous vehicles.
+  - **Denso Corporation**: Known for developing various types of sensors used in autonomous driving technologies, such as cameras and radar units.</t>
         </is>
       </c>
       <c r="I7" t="b">
@@ -2107,12 +2235,12 @@
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:52.484120Z</t>
+          <t>2026-03-23T18:47:01.422277Z</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1860.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2830.0}</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -2123,7 +2251,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2158,11 +2286,14 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>- Battery cells and modules have high supplier concentration risks due to limited production facilities in the region.
-- Electric motors face similar challenges, with few manufacturers specializing in their production.
-- Power electronics and management systems also exhibit significant supply chain risks because of a lack of local suppliers.
-- Rare earth materials used in EV components are at risk due to reliance on imports from China.
-- Lithium-ion battery raw materials present high concentration risks owing to limited regional sourcing options.</t>
+          <t>- Battery cells and modules often exhibit high supplier concentration due to limited manufacturing capacity globally, which is also true for the Southeast region of the United States.
+- Electric motors and power electronics may have concentrated supply chains if a few dominant manufacturers control production.
+- Rare earth metals used in EV components are typically sourced from a small number of global suppliers, increasing risk.
+- Lithium-ion battery raw materials (e.g., lithium, cobalt) often come from limited geographical sources, creating concentration risks.
+- Charging infrastructure components might face supply chain risks if major charging network providers dominate the Southeast market.
+Illustrative examples:
+- Tier 1: Battery cell manufacturers like Panasonic or LG Energy Solution
+- Tier 2: Rare earth metal suppliers such as Molycorp (USA)</t>
         </is>
       </c>
       <c r="I8" t="b">
@@ -2171,12 +2302,12 @@
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:54.202886Z</t>
+          <t>2026-03-23T18:47:04.189278Z</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1720.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2770.0}</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -2187,7 +2318,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2222,12 +2353,13 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>- Many electric vehicle (EV) manufacturers rely heavily on imported lithium from countries like Chile, Australia, and China for battery production.
-- Cobalt, another critical component in batteries, is predominantly sourced from the Democratic Republic of Congo due to its rich deposits.
-- Supply chain disruptions in these regions can significantly impact battery manufacturing capacity globally.
-- The geopolitical tensions between major importing nations and exporting countries affect supply stability and pricing.
-- Diversification efforts are underway by companies to secure alternative sources and reduce dependency on single-country imports.
-- Recycling initiatives for spent batteries aim to create a more sustainable and less dependent supply chain in the long term.</t>
+          <t>- **Raw Material Imports**: Many countries rely heavily on imported raw materials such as lithium, cobalt, and nickel from countries like Chile, Congo, and Indonesia for battery production.
+- **Manufacturing Components**: Battery manufacturing often requires specialized components that may be sourced internationally due to technological or logistical advantages in certain regions.
+- **Technological Dependencies**: Advanced technologies used in battery production might come from leading technology hubs such as South Korea (LG Chem) or Japan (Panasonic), which can influence supply chain dynamics.
+- **Logistical Challenges**: International shipping and logistics play a critical role, with potential disruptions due to geopolitical tensions, natural disasters, or pandemics affecting global trade routes.
+- **Regulatory Compliance**: Adherence to international regulations and standards is crucial for battery manufacturers, impacting sourcing decisions and operational costs.
+- **Tier 1 Suppliers**: Major players like China’s CATL (Contemporary Amperex Technology Ltd) and South Korea’s Samsung SDI are key suppliers in the global battery market.
+- **Tier 2 Suppliers**: Smaller but significant suppliers include companies that specialize in specific materials or components, such as Albemarle Corporation for lithium processing.</t>
         </is>
       </c>
       <c r="I9" t="b">
@@ -2236,12 +2368,12 @@
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:56.503286Z</t>
+          <t>2026-03-23T18:47:08.343936Z</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2300.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 4150.0}</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -2252,7 +2384,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2287,12 +2419,15 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>- Tier 2 and Tier 3 bottlenecks can significantly affect the supply chain efficiency of Original Equipment Manufacturers (OEMs).
-- Delays in obtaining components from Tier 2 suppliers can lead to reduced output at assembly lines, impacting overall production schedules.
-- Quality issues with Tier 3 parts can cascade up through the supply chain, causing rework and delays for OEMs.
-- Shortages or disruptions in raw materials supplied by Tier 3 vendors can limit the availability of critical components needed by Tier 2 suppliers.
-- Inflexible logistics from Tier 2 and Tier 3 suppliers can cause bottlenecks in inventory management at OEM facilities.
-- Communication breakdowns between lower-tier suppliers and OEMs can result in mismatches in production forecasts, leading to excess or shortage issues.</t>
+          <t>- **Supply Chain Disruptions:** Tier 2 and Tier 3 suppliers often have less robust supply chains, leading to potential disruptions that can affect the availability of critical components for OEMs.
+- **Quality Control Issues:** Smaller suppliers may lack advanced quality control measures, resulting in defective parts that delay production lines at OEM facilities.
+- **Capacity Constraints:** Limited manufacturing capacity at Tier 2 and Tier 3 vendors can cause bottlenecks when there is unexpected demand or sudden increases in orders from OEMs.
+- **Technological Limitations:** Smaller suppliers might not have the latest technology, leading to slower production times and inefficiencies that impact OEM schedules.
+- **Financial Instability:** Financial difficulties at lower-tier suppliers can lead to delayed deliveries or even bankruptcy, causing significant disruptions for OEMs.
+- **Logistical Challenges:** Tier 2 and Tier 3 companies often face logistical challenges such as transportation delays or storage issues, which can impede the timely delivery of parts to OEM production lines.
+Illustrative examples:
+- A small electronics manufacturer (Tier 3) facing a sudden shortage of raw materials due to global supply chain disruptions.
+- A medium-sized supplier (Tier 2) experiencing quality control failures that require extensive rework and delays in part deliveries.</t>
         </is>
       </c>
       <c r="I10" t="b">
@@ -2301,12 +2436,12 @@
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-03-23T18:20:59.393016Z</t>
+          <t>2026-03-23T18:47:12.893271Z</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2890.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 4550.0}</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -2317,7 +2452,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2352,11 +2487,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>- Battery manufacturing and recycling facilities are expanding rapidly due to proximity to automotive assembly plants.
-- Charging infrastructure installation companies are seeing significant growth as electric vehicle adoption increases.
-- Lithium-ion battery component suppliers are establishing regional hubs for quicker delivery times.
-- Electric vehicle (EV) service centers specializing in EV maintenance and repair are proliferating.
-- Regional distribution networks for EV parts and components are becoming more efficient and extensive.</t>
+          <t>- Battery manufacturing and recycling facilities are expanding rapidly due to increased demand for electric vehicles (EVs).
+- Charging infrastructure installation companies are seeing significant growth as more public charging stations are required to support EV adoption.
+- Lithium-ion battery component suppliers are experiencing strong growth, driven by the need for advanced materials in EV batteries.
+- Electric vehicle assembly plants are being established or expanded by major automakers looking to capitalize on regional incentives and supply chain proximity.
+- Tier 1 illustrative examples: Battery manufacturing (e.g., LG Energy Solution), Charging infrastructure providers (e.g., ChargePoint).
+- Tier 2 illustrative examples: Component suppliers for battery materials, Local charging station installation companies.</t>
         </is>
       </c>
       <c r="I11" t="b">
@@ -2365,12 +2501,12 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:00.957549Z</t>
+          <t>2026-03-23T18:47:15.401453Z</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 1560.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2510.0}</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -2381,7 +2517,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2416,11 +2552,11 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>- Volkswagen has committed significant resources to electric vehicle production and is phasing out traditional internal combustion engine (ICE) vehicles in many markets.
-- General Motors is investing heavily in battery technology and plans to launch multiple new electric models, reducing focus on conventional engines.
-- Ford Motor Company is expanding its EV lineup with the Mustang Mach-E and F-150 Lightning while scaling back some ICE vehicle production lines.
-- Toyota has announced a shift towards hybrid and fully electric vehicles as part of its long-term strategy, though it continues to support traditional ICE technology in certain markets.
-- Hyundai-Kia is rapidly growing its portfolio of electric cars and plans substantial investments in battery manufacturing facilities.</t>
+          <t>- Automotive giants like General Motors and Volkswagen are transitioning their product lines towards electric vehicles (EVs), phasing out internal combustion engine (ICE) components.
+- Suppliers such as Bosch and Continental are adapting by developing new technologies for EVs, including battery management systems and electric drivetrains.
+- Startups focused on EV technology, such as Rivian and Lucid Motors, are gaining traction and influencing established companies to shift their focus towards EV products.
+- Traditional ICE component manufacturers like Delphi Technologies are rebranding and restructuring to emphasize their role in the EV supply chain.
+- Companies like Panasonic, which have a strong presence in battery manufacturing for consumer electronics, are expanding into automotive batteries for EVs.</t>
         </is>
       </c>
       <c r="I12" t="b">
@@ -2429,12 +2565,12 @@
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:03.409028Z</t>
+          <t>2026-03-23T18:47:17.976334Z</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2450.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2570.0}</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -2445,7 +2581,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2480,12 +2616,14 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>- Demand for battery manufacturing equipment is increasing in Asia due to the rapid growth of electric vehicle (EV) markets and government incentives in countries like China and South Korea.
-- Europe is also seeing significant growth, driven by ambitious climate goals and investments from major automakers such as Volkswagen and BMW.
-- North America is experiencing strong demand, particularly in the United States, where there are substantial federal and state-level initiatives to support EV infrastructure and battery production.
-- Latin American countries like Brazil and Chile are showing interest due to their rich lithium reserves and growing automotive industries.
-- In Africa, regions with significant mineral resources are attracting investments for battery manufacturing as global supply chains diversify.
-- Middle Eastern nations are exploring opportunities in battery manufacturing to reduce reliance on oil exports and capitalize on renewable energy initiatives.</t>
+          <t>- Demand for battery manufacturing equipment is increasing in regions with significant investments in electric vehicle (EV) and renewable energy sectors, such as Asia-Pacific, Europe, and North America.
+- China has seen a surge in demand due to government incentives supporting EV production and storage solutions.
+- The European Union is focusing on localizing battery production to reduce reliance on imports and meet ambitious climate goals.
+- In the United States, states like California and Michigan are experiencing high demand as automakers expand their EV manufacturing capabilities.
+- South Korea and Japan are also seeing increased demand due to established electronics and automotive industries investing in advanced battery technologies.
+- Illustrative examples of regions with growing demand include:
+  - Tier 1: Asia-Pacific (China, South Korea)
+  - Tier 2: Europe (Germany, Poland), North America (California, Michigan)</t>
         </is>
       </c>
       <c r="I13" t="b">
@@ -2494,12 +2632,12 @@
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:06.279677Z</t>
+          <t>2026-03-23T18:47:21.001963Z</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2870.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 3030.0}</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -2510,7 +2648,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2545,11 +2683,13 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>- Miami-Dade County, Florida: High concentration of electric vehicle (EV) suppliers and a large workforce in the automotive industry.
-- Orange County, Florida: Presence of EV charging infrastructure companies and significant employment opportunities in tech and manufacturing sectors.
-- Harris County, Texas: Home to multiple EV component manufacturers and a robust labor market with skilled workers.
-- Maricopa County, Arizona: Growing presence of EV startups and established suppliers, along with a trainable workforce due to local educational institutions.
-- Clark County, Nevada: Increasing number of EV-related businesses and a growing tech-savvy workforce.</t>
+          <t>- Counties in the Southeastern United States that are likely to have high electric vehicle (EV) supplier density and a robust workforce include those near major automotive manufacturing hubs.
+- Illustrative examples of such counties might be:
+  - Shelby County, Alabama: Home to Ford Motor Company’s River Rouge Complex, which has shown interest in EV production.
+  - Greenville County, South Carolina: Known for its strong automotive industry presence, including BMW's plant and numerous suppliers.
+- These areas typically have established infrastructure and a skilled workforce trained in manufacturing processes relevant to EV production.
+- Counties with universities or technical colleges that offer specialized training programs related to automotive engineering and technology are also likely candidates.
+- Tier 1 counties would be those directly adjacent to major automotive plants, while Tier 2 might include nearby counties with significant supplier networks but slightly less direct plant proximity.</t>
         </is>
       </c>
       <c r="I14" t="b">
@@ -2558,12 +2698,12 @@
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:08.470736Z</t>
+          <t>2026-03-23T18:47:24.072727Z</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2190.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 3070.0}</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -2574,7 +2714,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2609,11 +2749,11 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>- Southeast Asia: Countries like Thailand, Vietnam, and Indonesia have emerging automotive industries with supportive government policies for electric vehicle (EV) manufacturing.
-- North America: The United States has a robust industrial base and a growing EV market, supported by local supply chains and favorable tax incentives.
-- Europe: Germany and Poland offer established manufacturing ecosystems along with proximity to major car manufacturers and battery suppliers like CATL and LG Energy Solution.
-- China: Despite potential trade barriers, it remains the world's largest EV market with extensive supplier networks and technological advancements in battery technology.
-- South Korea: Home to leading battery companies such as Samsung SDI and LG Chem, providing a strong local supply chain for battery pack assembly.</t>
+          <t>- **Tier 1 Regions:** Areas with established automotive manufacturing hubs, robust supply chains, and favorable government policies supporting electric vehicle (EV) production.
+- **Tier 2 Regions:** Locations that are emerging in the EV sector but may lack some of the mature infrastructure found in Tier 1 regions.
+**Illustrative Examples:**
+- **Southeastern United States:** Tennessee, with its strong automotive industry presence around Nashville and Memphis, and Alabama, home to major automotive manufacturing facilities.
+- **East Asia:** South Korea’s Ulsan region, known for its concentration of automotive manufacturers and suppliers.</t>
         </is>
       </c>
       <c r="I15" t="b">
@@ -2622,12 +2762,12 @@
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:11.035835Z</t>
+          <t>2026-03-23T18:47:26.306040Z</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2560.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2230.0}</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -2638,7 +2778,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>20260323T182038Z_qwen14b_no_rag</t>
+          <t>20260323T184634Z_qwen14b_no_rag</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2673,11 +2813,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>- Rural areas in China are seeing the growth of electric vehicle (EV) manufacturing due to government incentives and infrastructure development.
-- Small cities and towns in India are becoming hubs for EV production as local demand increases and startups enter the market.
-- Eastern European countries like Romania and Bulgaria are attracting EV manufacturers with lower operational costs and supportive policies.
-- In North America, smaller cities such as Windsor, Ontario (near Detroit), are leveraging existing automotive industry infrastructure to develop EV manufacturing capabilities.
-- South Korea is expanding its EV production beyond Seoul and Busan, with new plants being established in secondary cities like Daejeon and Gwangju.</t>
+          <t>- Emerging electric vehicle (EV) manufacturing clusters can be found in smaller cities and rural areas that offer lower operational costs, abundant land for factory sites, and supportive local policies. 
+- For example, the U.S. state of Michigan has seen growth in EV manufacturing beyond Detroit, with companies establishing plants in cities like Holland.
+- Another illustrative example is the city of Sunderland in the UK, where Nissan established an EV production facility outside London and other major metropolitan areas.
+- Tier 1 locations would be smaller industrial or suburban towns near existing automotive supply chains but with lower real estate costs. 
+- Tier 2 locations might include rural regions that offer tax incentives for green manufacturing initiatives.
+- These clusters often benefit from government grants, research partnerships with local universities, and a skilled workforce trained in traditional automotive industries.</t>
         </is>
       </c>
       <c r="I16" t="b">
@@ -2686,12 +2827,12 @@
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-03-23T18:21:13.371844Z</t>
+          <t>2026-03-23T18:47:29.255100Z</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2340.0}</t>
+          <t>{'retrieval_ms_local': 0.0, 'retrieval_ms_tavily': 0.0, 'generation_ms': 2950.0}</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>

</xml_diff>